<commit_message>
feat: update task management with new timeline fields and color scheme
- Added `uatDate` and `prdDate` fields to task model and forms.
- Updated color scheme to use new primary color `#6BB82A` across the application.
- Adjusted related documentation and styles to reflect the new theme and task attributes.
- Modified navigation to redirect to the dashboard instead of projects.
</commit_message>
<xml_diff>
--- a/data/taskDB.xlsx
+++ b/data/taskDB.xlsx
@@ -589,7 +589,7 @@
         <v>2026-09-01T07:23:24.979Z</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-09-04T07:27:25.696Z</v>
+        <v>2026-09-04T07:56:38.400Z</v>
       </c>
     </row>
     <row r="3">
@@ -609,7 +609,7 @@
         <v>2026-09-01T07:23:24.981Z</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-09-04T07:27:25.703Z</v>
+        <v>2026-09-04T07:56:38.404Z</v>
       </c>
     </row>
     <row r="4">
@@ -629,7 +629,7 @@
         <v>2026-09-01T07:23:24.983Z</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-09-04T07:27:11.500Z</v>
+        <v>2026-09-04T07:56:38.422Z</v>
       </c>
     </row>
     <row r="5">
@@ -649,7 +649,7 @@
         <v>2026-09-01T07:23:24.985Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-04T07:20:50.970Z</v>
+        <v>2026-09-04T07:56:38.414Z</v>
       </c>
     </row>
     <row r="6">
@@ -660,7 +660,7 @@
         <v>Done</v>
       </c>
       <c r="C6" t="str">
-        <v>#1E3A5F</v>
+        <v>#6BB82A</v>
       </c>
       <c r="D6" t="str">
         <v>2</v>
@@ -669,7 +669,7 @@
         <v>2026-09-01T07:23:24.988Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-04T07:20:50.968Z</v>
+        <v>2026-09-04T07:56:38.410Z</v>
       </c>
     </row>
     <row r="7">
@@ -758,7 +758,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:P1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -783,30 +783,36 @@
         <v>endDate</v>
       </c>
       <c r="H1" t="str">
+        <v>uatDate</v>
+      </c>
+      <c r="I1" t="str">
+        <v>prdDate</v>
+      </c>
+      <c r="J1" t="str">
         <v>sortOrder</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>projectId</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>priorityId</v>
       </c>
-      <c r="K1" t="str">
+      <c r="M1" t="str">
         <v>statusId</v>
       </c>
-      <c r="L1" t="str">
+      <c r="N1" t="str">
         <v>assigneeId</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>createdAt</v>
       </c>
-      <c r="N1" t="str">
+      <c r="P1" t="str">
         <v>updatedAt</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: enhance task management with new task types and subtasks
- Introduced new models for TaskType and Subtask in the database schema.
- Updated task forms and views to support multiple task types and subtasks.
- Enhanced API endpoints for creating, updating, and deleting task types and subtasks.
- Modified UI components to display task types and subtasks effectively across the application.
- Updated existing task management logic to accommodate the new features.
</commit_message>
<xml_diff>
--- a/data/taskDB.xlsx
+++ b/data/taskDB.xlsx
@@ -9,6 +9,9 @@
     <sheet name="TeamMembers" sheetId="4" r:id="rId4"/>
     <sheet name="Tasks" sheetId="5" r:id="rId5"/>
     <sheet name="StatusHistories" sheetId="6" r:id="rId6"/>
+    <sheet name="Subtasks" sheetId="7" r:id="rId7"/>
+    <sheet name="TaskAssignees" sheetId="8" r:id="rId8"/>
+    <sheet name="TaskTypes" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -589,7 +592,7 @@
         <v>2026-09-01T07:23:24.979Z</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-09-04T07:56:38.400Z</v>
+        <v>2026-09-04T08:58:01.411Z</v>
       </c>
     </row>
     <row r="3">
@@ -609,7 +612,7 @@
         <v>2026-09-01T07:23:24.981Z</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-09-04T07:56:38.404Z</v>
+        <v>2026-09-04T08:58:01.417Z</v>
       </c>
     </row>
     <row r="4">
@@ -629,7 +632,7 @@
         <v>2026-09-01T07:23:24.983Z</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-09-04T07:56:38.422Z</v>
+        <v>2026-09-04T08:58:01.424Z</v>
       </c>
     </row>
     <row r="5">
@@ -649,7 +652,7 @@
         <v>2026-09-01T07:23:24.985Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-04T07:56:38.414Z</v>
+        <v>2026-09-04T08:58:01.421Z</v>
       </c>
     </row>
     <row r="6">
@@ -669,7 +672,7 @@
         <v>2026-09-01T07:23:24.988Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-04T07:56:38.410Z</v>
+        <v>2026-09-04T08:58:01.419Z</v>
       </c>
     </row>
     <row r="7">
@@ -701,7 +704,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -749,9 +752,170 @@
         <v>2026-09-01T07:26:41.854Z</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ครีม</v>
+      </c>
+      <c r="C3" t="str">
+        <v>#EF4444</v>
+      </c>
+      <c r="D3" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="E3" t="str">
+        <v>1</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-09-04T08:31:09.214Z</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-09-04T08:31:09.214Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+      </c>
+      <c r="B4" t="str">
+        <v>พี่เอก</v>
+      </c>
+      <c r="C4" t="str">
+        <v>#F97316</v>
+      </c>
+      <c r="D4" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-09-04T08:31:15.973Z</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-09-04T08:31:15.973Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+      </c>
+      <c r="B5" t="str">
+        <v>พี่จู</v>
+      </c>
+      <c r="C5" t="str">
+        <v>#3B82F6</v>
+      </c>
+      <c r="D5" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="E5" t="str">
+        <v>3</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-09-04T08:31:24.760Z</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-09-04T08:31:24.760Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
+      </c>
+      <c r="B6" t="str">
+        <v>ตาเฟม</v>
+      </c>
+      <c r="C6" t="str">
+        <v>#8B5CF6</v>
+      </c>
+      <c r="D6" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="E6" t="str">
+        <v>4</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-09-04T08:31:29.670Z</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-09-04T08:31:29.670Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="B7" t="str">
+        <v>มาย</v>
+      </c>
+      <c r="C7" t="str">
+        <v>#EC4899</v>
+      </c>
+      <c r="D7" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="E7" t="str">
+        <v>5</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-09-04T08:31:33.588Z</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-09-04T08:31:33.588Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="B8" t="str">
+        <v>บรีส</v>
+      </c>
+      <c r="C8" t="str">
+        <v>#75D7F0</v>
+      </c>
+      <c r="D8" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="E8" t="str">
+        <v>6</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-09-04T08:31:52.262Z</v>
+      </c>
+      <c r="G8" t="str">
+        <v>2026-09-04T08:31:52.262Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>190c2d73-d236-4277-a3e1-b6004555ac94</v>
+      </c>
+      <c r="B9" t="str">
+        <v>พริ้ง</v>
+      </c>
+      <c r="C9" t="str">
+        <v>#F0EC75</v>
+      </c>
+      <c r="D9" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="E9" t="str">
+        <v>7</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-09-04T08:32:04.538Z</v>
+      </c>
+      <c r="G9" t="str">
+        <v>2026-09-04T08:32:04.538Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -855,4 +1019,140 @@
     <ignoredError numberStoredAsText="1" sqref="A1:I1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>taskId</v>
+      </c>
+      <c r="C1" t="str">
+        <v>name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>isDone</v>
+      </c>
+      <c r="E1" t="str">
+        <v>sortOrder</v>
+      </c>
+      <c r="F1" t="str">
+        <v>createdAt</v>
+      </c>
+      <c r="G1" t="str">
+        <v>updatedAt</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>taskId</v>
+      </c>
+      <c r="C1" t="str">
+        <v>teamMemberId</v>
+      </c>
+      <c r="D1" t="str">
+        <v>sortOrder</v>
+      </c>
+      <c r="E1" t="str">
+        <v>createdAt</v>
+      </c>
+      <c r="F1" t="str">
+        <v>updatedAt</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>color</v>
+      </c>
+      <c r="D1" t="str">
+        <v>sortOrder</v>
+      </c>
+      <c r="E1" t="str">
+        <v>createdAt</v>
+      </c>
+      <c r="F1" t="str">
+        <v>updatedAt</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>550e258b-aefd-44cc-988f-844559da921f</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="C2" t="str">
+        <v>#3B82F6</v>
+      </c>
+      <c r="D2" t="str">
+        <v>0</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-09-04T08:58:01.426Z</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-09-04T08:58:01.426Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>d3762279-50c6-4edc-a73d-66468851222f</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Front End</v>
+      </c>
+      <c r="C3" t="str">
+        <v>#EC4899</v>
+      </c>
+      <c r="D3" t="str">
+        <v>1</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-09-04T08:58:01.430Z</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-09-04T08:58:01.430Z</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: update taskDB.xlsx with new data
</commit_message>
<xml_diff>
--- a/data/taskDB.xlsx
+++ b/data/taskDB.xlsx
@@ -922,7 +922,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -974,16 +974,916 @@
         <v>updatedAt</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>d6acd7ea-e69f-4894-9ce4-c8ae86da6bd2</v>
+      </c>
+      <c r="B2" t="str">
+        <v>กรมธรรม์</v>
+      </c>
+      <c r="C2" t="str">
+        <v xml:space="preserve"> มติ 14 กรกฎาคม 2569</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="J2" t="str">
+        <v>0</v>
+      </c>
+      <c r="K2" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L2" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M2" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="N2" t="str">
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
+      </c>
+      <c r="O2" t="str">
+        <v>2026-09-04T09:22:21.943Z</v>
+      </c>
+      <c r="P2" t="str">
+        <v>2026-09-04T09:42:39.373Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
+      </c>
+      <c r="B3" t="str">
+        <v>แจ้งเตือน</v>
+      </c>
+      <c r="C3" t="str">
+        <v>กดรายการแจ้งเตือน ให้ลิงก์ไปยังหน้าจัดการข้อมูลที่แจ้งเตือนได้</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>Back End, Front End</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="J3" t="str">
+        <v>0</v>
+      </c>
+      <c r="K3" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L3" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M3" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="N3" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="O3" t="str">
+        <v>2026-09-04T09:24:04.693Z</v>
+      </c>
+      <c r="P3" t="str">
+        <v>2026-09-04T09:42:32.107Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
+      </c>
+      <c r="B4" t="str">
+        <v>เคลม</v>
+      </c>
+      <c r="C4" t="str">
+        <v>เมนูตั้งค่ายา (TMT) (แก้ไขเพิ่มเติม)</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>Back End, Front End</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="J4" t="str">
+        <v>0</v>
+      </c>
+      <c r="K4" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L4" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M4" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="N4" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="O4" t="str">
+        <v>2026-09-04T09:24:33.365Z</v>
+      </c>
+      <c r="P4" t="str">
+        <v>2026-09-04T09:42:23.325Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
+      </c>
+      <c r="B5" t="str">
+        <v>กรมธรรม์</v>
+      </c>
+      <c r="C5" t="str">
+        <v>กรมธรรม์ มติ 14 กรกฎาคม 2569 - แก้ไขบั๊คเช็คผู้ปกครองเด็ก</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-09-01</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>2026-09-01</v>
+      </c>
+      <c r="J5" t="str">
+        <v>0</v>
+      </c>
+      <c r="K5" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L5" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M5" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="N5" t="str">
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
+      </c>
+      <c r="O5" t="str">
+        <v>2026-09-04T09:25:10.002Z</v>
+      </c>
+      <c r="P5" t="str">
+        <v>2026-09-04T09:42:08.479Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
+      </c>
+      <c r="B6" t="str">
+        <v>STM &amp; รายงาน</v>
+      </c>
+      <c r="C6" t="str">
+        <v>รายงาน ค1(1) (Portal และ Excel)</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v>Back End, Front End</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-09-02</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2026-09-02</v>
+      </c>
+      <c r="I6" t="str">
+        <v>2026-09-02</v>
+      </c>
+      <c r="J6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K6" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L6" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M6" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="N6" t="str">
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+      </c>
+      <c r="O6" t="str">
+        <v>2026-09-04T09:26:00.676Z</v>
+      </c>
+      <c r="P6" t="str">
+        <v>2026-09-04T09:42:00.055Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+      </c>
+      <c r="B7" t="str">
+        <v>ใบรับรองแพทย์</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v>Front End</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="H7" t="str">
+        <v>2026-09-02</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v>0</v>
+      </c>
+      <c r="K7" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L7" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M7" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="N7" t="str">
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+      </c>
+      <c r="O7" t="str">
+        <v>2026-09-04T09:27:00.612Z</v>
+      </c>
+      <c r="P7" t="str">
+        <v>2026-09-04T09:40:57.950Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>1e95dc95-6f63-4810-9d57-8520eb9b42c5</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Export ผลตรวจสุขภาพ</v>
+      </c>
+      <c r="C8" t="str">
+        <v>เพิ่มข้อมูล Fcode</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G8" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="H8" t="str">
+        <v>2026-09-02</v>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v>0</v>
+      </c>
+      <c r="K8" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L8" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M8" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="N8" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="O8" t="str">
+        <v>2026-09-04T09:29:47.993Z</v>
+      </c>
+      <c r="P8" t="str">
+        <v>2026-09-04T09:41:39.538Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
+      </c>
+      <c r="B9" t="str">
+        <v>เอกสารเลขอ้างอิง และสร้างเอกสารใหม่หลังออกเลขอ้างอิง</v>
+      </c>
+      <c r="C9" t="str">
+        <v>แยกงวดกรมธรรม์กรณีมีหลายงวด</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v>Back End, Front End</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G9" t="str">
+        <v>2026-09-02</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v>2026-09-02</v>
+      </c>
+      <c r="J9" t="str">
+        <v>0</v>
+      </c>
+      <c r="K9" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L9" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M9" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="N9" t="str">
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+      </c>
+      <c r="O9" t="str">
+        <v>2026-09-04T09:32:18.156Z</v>
+      </c>
+      <c r="P9" t="str">
+        <v>2026-09-04T09:41:51.999Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>62533ab0-8ef1-45b9-b2d4-961570759b92</v>
+      </c>
+      <c r="B10" t="str">
+        <v>iFrame for HIS</v>
+      </c>
+      <c r="C10" t="str">
+        <v>ตรวจสอบยืนยันตัวตนผ่านระบบ Bio ID (ใบหน้า และม่านตา)</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v>Back End, Front End</v>
+      </c>
+      <c r="F10" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="H10" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v>0</v>
+      </c>
+      <c r="K10" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L10" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M10" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="N10" t="str">
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+      </c>
+      <c r="O10" t="str">
+        <v>2026-09-04T09:33:03.132Z</v>
+      </c>
+      <c r="P10" t="str">
+        <v>2026-09-04T09:40:43.627Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>e0e2d398-49d2-4dc3-9fbc-512e2b97e4f5</v>
+      </c>
+      <c r="B11" t="str">
+        <v>กรมธรรม์</v>
+      </c>
+      <c r="C11" t="str">
+        <v>เพิม Filter ชือกรมธรรม์ (ใช้ชื่อตามรายงานส่งเงิน)</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F11" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="H11" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v>0</v>
+      </c>
+      <c r="K11" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L11" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M11" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="N11" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="O11" t="str">
+        <v>2026-09-04T09:33:38.656Z</v>
+      </c>
+      <c r="P11" t="str">
+        <v>2026-09-04T09:41:08.425Z</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>a4db697d-4d50-4200-8355-647ab86cd480</v>
+      </c>
+      <c r="B12" t="str">
+        <v>ส่งเคลม</v>
+      </c>
+      <c r="C12" t="str">
+        <v>เงื่อนไขการส่งเคลมหมวด 8</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F12" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G12" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v>0</v>
+      </c>
+      <c r="K12" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L12" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M12" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="N12" t="str">
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+      </c>
+      <c r="O12" t="str">
+        <v>2026-09-04T09:34:04.072Z</v>
+      </c>
+      <c r="P12" t="str">
+        <v>2026-09-04T09:40:35.751Z</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>12f8c884-7a9e-4086-8352-ace2ea778248</v>
+      </c>
+      <c r="B13" t="str">
+        <v>LogReport ฝั่งกองทุน</v>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F13" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="G13" t="str">
+        <v>2026-09-09</v>
+      </c>
+      <c r="H13" t="str">
+        <v>2026-09-09</v>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v>0</v>
+      </c>
+      <c r="K13" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L13" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M13" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="N13" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="O13" t="str">
+        <v>2026-09-04T09:43:36.886Z</v>
+      </c>
+      <c r="P13" t="str">
+        <v>2026-09-04T09:45:31.790Z</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
+      </c>
+      <c r="B14" t="str">
+        <v>LogReport ส่งเคลม</v>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F14" t="str">
+        <v>2026-08-24</v>
+      </c>
+      <c r="G14" t="str">
+        <v>2026-09-09</v>
+      </c>
+      <c r="H14" t="str">
+        <v>2026-09-09</v>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v>0</v>
+      </c>
+      <c r="K14" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L14" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M14" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="N14" t="str">
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+      </c>
+      <c r="O14" t="str">
+        <v>2026-09-04T09:43:56.520Z</v>
+      </c>
+      <c r="P14" t="str">
+        <v>2026-09-04T09:45:22.510Z</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
+      </c>
+      <c r="B15" t="str">
+        <v>เปลี่ยนสิทธิ/ยกเลิกสิทธิ</v>
+      </c>
+      <c r="C15" t="str">
+        <v>เพิ่มค้นหาด้วยเลขอ้างอิง พร้อมเลือกทำรายการได้หลายรายการพร้อมกัน + เปลี่ยนการแสดงผลหน้าค้นหา</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F15" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="G15" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="H15" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v>0</v>
+      </c>
+      <c r="K15" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L15" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M15" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="N15" t="str">
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+      </c>
+      <c r="O15" t="str">
+        <v>2026-09-04T09:44:42.509Z</v>
+      </c>
+      <c r="P15" t="str">
+        <v>2026-09-04T09:44:49.331Z</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
+      </c>
+      <c r="B16" t="str">
+        <v>STM &amp; รายงาน</v>
+      </c>
+      <c r="C16" t="str">
+        <v>อยากให้นำเข้าไฟล์ 1 ไฟล์ได้หลายวัน / เลือกไฟล์ได้มากกว่า 1 ไฟล์ต่อนำเข้า 1 ครั้ง</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v>Back End, Front End</v>
+      </c>
+      <c r="F16" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G16" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="H16" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v>0</v>
+      </c>
+      <c r="K16" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L16" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M16" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="N16" t="str">
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+      </c>
+      <c r="O16" t="str">
+        <v>2026-09-04T09:47:39.827Z</v>
+      </c>
+      <c r="P16" t="str">
+        <v>2026-09-04T09:47:39.843Z</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
+      </c>
+      <c r="B17" t="str">
+        <v>รายงานย้ายสิทธิ</v>
+      </c>
+      <c r="C17" t="str">
+        <v>เพิ่ม filter รพ ปลายทาง + บั๊ค</v>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v>Back End, Front End</v>
+      </c>
+      <c r="F17" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G17" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="H17" t="str">
+        <v>2026-09-16</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v>0</v>
+      </c>
+      <c r="K17" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L17" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M17" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="N17" t="str">
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+      </c>
+      <c r="O17" t="str">
+        <v>2026-09-04T09:48:58.057Z</v>
+      </c>
+      <c r="P17" t="str">
+        <v>2026-09-04T09:48:58.073Z</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
+      </c>
+      <c r="B18" t="str">
+        <v>LogReport</v>
+      </c>
+      <c r="C18" t="str">
+        <v xml:space="preserve"> Log ใบรับรองแพทย์ Collection ใหม่ ,ปรับ Log กรมธรรม์ไปใช้ Collection ใหม่</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F18" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G18" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="H18" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v>0</v>
+      </c>
+      <c r="K18" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L18" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M18" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="N18" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="O18" t="str">
+        <v>2026-09-04T09:50:04.917Z</v>
+      </c>
+      <c r="P18" t="str">
+        <v>2026-09-04T09:50:04.931Z</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+      </c>
+      <c r="B19" t="str">
+        <v>LogReport</v>
+      </c>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v>Back End</v>
+      </c>
+      <c r="F19" t="str">
+        <v>2026-08-31</v>
+      </c>
+      <c r="G19" t="str">
+        <v>2026-09-25</v>
+      </c>
+      <c r="H19" t="str">
+        <v>2026-09-25</v>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v>0</v>
+      </c>
+      <c r="K19" t="str">
+        <v>6646c3f5-c7ec-4e87-bd40-a6a8fd0fccf3</v>
+      </c>
+      <c r="L19" t="str">
+        <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
+      </c>
+      <c r="M19" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="N19" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="O19" t="str">
+        <v>2026-09-04T09:51:03.522Z</v>
+      </c>
+      <c r="P19" t="str">
+        <v>2026-09-04T09:54:48.379Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P19"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I32"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1014,16 +1914,915 @@
         <v>updatedAt</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>0eab7894-0aec-485c-83c1-8bcf9a56a710</v>
+      </c>
+      <c r="B2" t="str">
+        <v>d6acd7ea-e69f-4894-9ce4-c8ae86da6bd2</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-09-04T09:22:21.958Z</v>
+      </c>
+      <c r="H2" t="str">
+        <v>2026-09-04T09:22:21.959Z</v>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-09-04T09:22:21.959Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>5a8e7b98-34e1-4b8d-a0d0-9ee92d9edd3f</v>
+      </c>
+      <c r="B3" t="str">
+        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-09-04T09:24:04.708Z</v>
+      </c>
+      <c r="H3" t="str">
+        <v>2026-09-04T09:24:04.709Z</v>
+      </c>
+      <c r="I3" t="str">
+        <v>2026-09-04T09:24:04.709Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>28747716-ac45-4bfb-8799-c59738ae14de</v>
+      </c>
+      <c r="B4" t="str">
+        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-09-04T09:24:33.384Z</v>
+      </c>
+      <c r="H4" t="str">
+        <v>2026-09-04T09:24:33.385Z</v>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-09-04T09:24:33.385Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>9bd840d4-b2f4-43b3-b21c-1b2850d48e75</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-09-04T09:25:10.021Z</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2026-09-04T09:25:10.022Z</v>
+      </c>
+      <c r="I5" t="str">
+        <v>2026-09-04T09:25:10.022Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>dda1a7fd-e261-417e-bc87-4b1c6741a812</v>
+      </c>
+      <c r="B6" t="str">
+        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-09-04T09:26:00.694Z</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2026-09-04T09:26:00.695Z</v>
+      </c>
+      <c r="I6" t="str">
+        <v>2026-09-04T09:26:00.695Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>25e63386-bce5-4998-8870-2419241bf3ef</v>
+      </c>
+      <c r="B7" t="str">
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-09-04T09:27:00.635Z</v>
+      </c>
+      <c r="H7" t="str">
+        <v>2026-09-04T09:27:00.635Z</v>
+      </c>
+      <c r="I7" t="str">
+        <v>2026-09-04T09:27:00.635Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>d4f8f326-ea07-463e-9600-ac447a9f7cce</v>
+      </c>
+      <c r="B8" t="str">
+        <v>1e95dc95-6f63-4810-9d57-8520eb9b42c5</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G8" t="str">
+        <v>2026-09-04T09:29:48.010Z</v>
+      </c>
+      <c r="H8" t="str">
+        <v>2026-09-04T09:29:48.012Z</v>
+      </c>
+      <c r="I8" t="str">
+        <v>2026-09-04T09:29:48.012Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>1f68e3ea-4f20-4152-bfe3-a531a2938fb5</v>
+      </c>
+      <c r="B9" t="str">
+        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G9" t="str">
+        <v>2026-09-04T09:32:18.175Z</v>
+      </c>
+      <c r="H9" t="str">
+        <v>2026-09-04T09:32:18.176Z</v>
+      </c>
+      <c r="I9" t="str">
+        <v>2026-09-04T09:32:18.176Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>60574bb6-d397-4be0-a022-53f307ecca67</v>
+      </c>
+      <c r="B10" t="str">
+        <v>62533ab0-8ef1-45b9-b2d4-961570759b92</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2026-09-04T09:33:03.148Z</v>
+      </c>
+      <c r="H10" t="str">
+        <v>2026-09-04T09:33:03.149Z</v>
+      </c>
+      <c r="I10" t="str">
+        <v>2026-09-04T09:33:03.149Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>a6333610-8aa8-44ff-aca8-04751afda114</v>
+      </c>
+      <c r="B11" t="str">
+        <v>e0e2d398-49d2-4dc3-9fbc-512e2b97e4f5</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2026-09-04T09:33:38.672Z</v>
+      </c>
+      <c r="H11" t="str">
+        <v>2026-09-04T09:33:38.673Z</v>
+      </c>
+      <c r="I11" t="str">
+        <v>2026-09-04T09:33:38.673Z</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>c645328c-ce34-465b-a2c9-3dd037a2e984</v>
+      </c>
+      <c r="B12" t="str">
+        <v>a4db697d-4d50-4200-8355-647ab86cd480</v>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G12" t="str">
+        <v>2026-09-04T09:34:04.089Z</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2026-09-04T09:34:04.090Z</v>
+      </c>
+      <c r="I12" t="str">
+        <v>2026-09-04T09:34:04.090Z</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>8a87a2d1-64bd-4b45-b68c-235eb134861d</v>
+      </c>
+      <c r="B13" t="str">
+        <v>d6acd7ea-e69f-4894-9ce4-c8ae86da6bd2</v>
+      </c>
+      <c r="C13" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E13" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="F13" t="str">
+        <v>PRD</v>
+      </c>
+      <c r="G13" t="str">
+        <v>2026-09-04T09:34:59.204Z</v>
+      </c>
+      <c r="H13" t="str">
+        <v>2026-09-04T09:34:59.205Z</v>
+      </c>
+      <c r="I13" t="str">
+        <v>2026-09-04T09:34:59.205Z</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>5d93951c-863e-41e7-a150-6180617b281e</v>
+      </c>
+      <c r="B14" t="str">
+        <v>a4db697d-4d50-4200-8355-647ab86cd480</v>
+      </c>
+      <c r="C14" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E14" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="F14" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="G14" t="str">
+        <v>2026-09-04T09:35:30.233Z</v>
+      </c>
+      <c r="H14" t="str">
+        <v>2026-09-04T09:35:30.235Z</v>
+      </c>
+      <c r="I14" t="str">
+        <v>2026-09-04T09:35:30.235Z</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>d7fde791-84cc-40b4-8f17-b30ed06feb28</v>
+      </c>
+      <c r="B15" t="str">
+        <v>e0e2d398-49d2-4dc3-9fbc-512e2b97e4f5</v>
+      </c>
+      <c r="C15" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E15" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="F15" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="G15" t="str">
+        <v>2026-09-04T09:35:49.810Z</v>
+      </c>
+      <c r="H15" t="str">
+        <v>2026-09-04T09:35:49.811Z</v>
+      </c>
+      <c r="I15" t="str">
+        <v>2026-09-04T09:35:49.811Z</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>be5c2d50-bd26-406e-a704-927d268b8de9</v>
+      </c>
+      <c r="B16" t="str">
+        <v>62533ab0-8ef1-45b9-b2d4-961570759b92</v>
+      </c>
+      <c r="C16" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E16" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="F16" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="G16" t="str">
+        <v>2026-09-04T09:35:55.095Z</v>
+      </c>
+      <c r="H16" t="str">
+        <v>2026-09-04T09:35:55.097Z</v>
+      </c>
+      <c r="I16" t="str">
+        <v>2026-09-04T09:35:55.097Z</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>ccc10e5c-cc02-4aae-84df-80c1cc71ca04</v>
+      </c>
+      <c r="B17" t="str">
+        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
+      </c>
+      <c r="C17" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E17" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="F17" t="str">
+        <v>PRD</v>
+      </c>
+      <c r="G17" t="str">
+        <v>2026-09-04T09:36:06.667Z</v>
+      </c>
+      <c r="H17" t="str">
+        <v>2026-09-04T09:36:06.668Z</v>
+      </c>
+      <c r="I17" t="str">
+        <v>2026-09-04T09:36:06.668Z</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>af113307-c54f-48cb-916c-65f644910f0b</v>
+      </c>
+      <c r="B18" t="str">
+        <v>1e95dc95-6f63-4810-9d57-8520eb9b42c5</v>
+      </c>
+      <c r="C18" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E18" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="F18" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="G18" t="str">
+        <v>2026-09-04T09:36:18.006Z</v>
+      </c>
+      <c r="H18" t="str">
+        <v>2026-09-04T09:36:18.010Z</v>
+      </c>
+      <c r="I18" t="str">
+        <v>2026-09-04T09:36:18.010Z</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>4656d424-49d4-43e7-ad48-71018ae53f45</v>
+      </c>
+      <c r="B19" t="str">
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+      </c>
+      <c r="C19" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E19" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="F19" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="G19" t="str">
+        <v>2026-09-04T09:36:27.699Z</v>
+      </c>
+      <c r="H19" t="str">
+        <v>2026-09-04T09:36:27.701Z</v>
+      </c>
+      <c r="I19" t="str">
+        <v>2026-09-04T09:36:27.701Z</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>ecb39be7-187e-45f2-9625-6670d47ae29d</v>
+      </c>
+      <c r="B20" t="str">
+        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
+      </c>
+      <c r="C20" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E20" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="F20" t="str">
+        <v>PRD</v>
+      </c>
+      <c r="G20" t="str">
+        <v>2026-09-04T09:36:34.985Z</v>
+      </c>
+      <c r="H20" t="str">
+        <v>2026-09-04T09:36:34.987Z</v>
+      </c>
+      <c r="I20" t="str">
+        <v>2026-09-04T09:36:34.987Z</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>cc76577e-f484-43c9-b465-c6dee07dc93b</v>
+      </c>
+      <c r="B21" t="str">
+        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
+      </c>
+      <c r="C21" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E21" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="F21" t="str">
+        <v>PRD</v>
+      </c>
+      <c r="G21" t="str">
+        <v>2026-09-04T09:36:40.481Z</v>
+      </c>
+      <c r="H21" t="str">
+        <v>2026-09-04T09:36:40.483Z</v>
+      </c>
+      <c r="I21" t="str">
+        <v>2026-09-04T09:36:40.483Z</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>3b38d2b1-1e4c-4e41-974a-fec89e2b565b</v>
+      </c>
+      <c r="B22" t="str">
+        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
+      </c>
+      <c r="C22" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E22" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="F22" t="str">
+        <v>PRD</v>
+      </c>
+      <c r="G22" t="str">
+        <v>2026-09-04T09:36:45.193Z</v>
+      </c>
+      <c r="H22" t="str">
+        <v>2026-09-04T09:36:45.195Z</v>
+      </c>
+      <c r="I22" t="str">
+        <v>2026-09-04T09:36:45.195Z</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>6fa966dd-4c68-4f1b-b4c4-3d71cd7223cc</v>
+      </c>
+      <c r="B23" t="str">
+        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
+      </c>
+      <c r="C23" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E23" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="F23" t="str">
+        <v>PRD</v>
+      </c>
+      <c r="G23" t="str">
+        <v>2026-09-04T09:36:49.384Z</v>
+      </c>
+      <c r="H23" t="str">
+        <v>2026-09-04T09:36:49.386Z</v>
+      </c>
+      <c r="I23" t="str">
+        <v>2026-09-04T09:36:49.386Z</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>72612f46-18dd-4fec-b1b1-a62dc1b92bb9</v>
+      </c>
+      <c r="B24" t="str">
+        <v>12f8c884-7a9e-4086-8352-ace2ea778248</v>
+      </c>
+      <c r="C24" t="str">
+        <v/>
+      </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G24" t="str">
+        <v>2026-09-04T09:43:36.905Z</v>
+      </c>
+      <c r="H24" t="str">
+        <v>2026-09-04T09:43:36.906Z</v>
+      </c>
+      <c r="I24" t="str">
+        <v>2026-09-04T09:43:36.906Z</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>eef1ce50-2385-4be1-8f35-b32237fded02</v>
+      </c>
+      <c r="B25" t="str">
+        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
+      </c>
+      <c r="C25" t="str">
+        <v/>
+      </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
+      <c r="E25" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G25" t="str">
+        <v>2026-09-04T09:43:56.539Z</v>
+      </c>
+      <c r="H25" t="str">
+        <v>2026-09-04T09:43:56.541Z</v>
+      </c>
+      <c r="I25" t="str">
+        <v>2026-09-04T09:43:56.541Z</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>fd98c168-e181-4df0-9fa1-2084a8618cc9</v>
+      </c>
+      <c r="B26" t="str">
+        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
+      </c>
+      <c r="C26" t="str">
+        <v/>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G26" t="str">
+        <v>2026-09-04T09:44:42.523Z</v>
+      </c>
+      <c r="H26" t="str">
+        <v>2026-09-04T09:44:42.525Z</v>
+      </c>
+      <c r="I26" t="str">
+        <v>2026-09-04T09:44:42.525Z</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>acc42cbd-f167-4f56-aa00-8f9b41d94c95</v>
+      </c>
+      <c r="B27" t="str">
+        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G27" t="str">
+        <v>2026-09-04T09:47:39.847Z</v>
+      </c>
+      <c r="H27" t="str">
+        <v>2026-09-04T09:47:39.849Z</v>
+      </c>
+      <c r="I27" t="str">
+        <v>2026-09-04T09:47:39.849Z</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>9c16f99b-8802-4522-9dd4-b482c02511ed</v>
+      </c>
+      <c r="B28" t="str">
+        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
+      </c>
+      <c r="C28" t="str">
+        <v/>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G28" t="str">
+        <v>2026-09-04T09:48:58.077Z</v>
+      </c>
+      <c r="H28" t="str">
+        <v>2026-09-04T09:48:58.078Z</v>
+      </c>
+      <c r="I28" t="str">
+        <v>2026-09-04T09:48:58.078Z</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>d6c9f656-2b17-4ade-b863-0702f8f5f0e4</v>
+      </c>
+      <c r="B29" t="str">
+        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
+      </c>
+      <c r="C29" t="str">
+        <v/>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G29" t="str">
+        <v>2026-09-04T09:50:04.935Z</v>
+      </c>
+      <c r="H29" t="str">
+        <v>2026-09-04T09:50:04.937Z</v>
+      </c>
+      <c r="I29" t="str">
+        <v>2026-09-04T09:50:04.937Z</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>3e78de04-3963-4bad-9dd2-06e4bec61a72</v>
+      </c>
+      <c r="B30" t="str">
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G30" t="str">
+        <v>2026-09-04T09:51:03.542Z</v>
+      </c>
+      <c r="H30" t="str">
+        <v>2026-09-04T09:51:03.543Z</v>
+      </c>
+      <c r="I30" t="str">
+        <v>2026-09-04T09:51:03.543Z</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>c343f0ff-91c4-4ce2-ad88-707ba5e8712a</v>
+      </c>
+      <c r="B31" t="str">
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+      </c>
+      <c r="C31" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="E31" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="F31" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="G31" t="str">
+        <v>2026-09-04T09:54:35.269Z</v>
+      </c>
+      <c r="H31" t="str">
+        <v>2026-09-04T09:54:35.271Z</v>
+      </c>
+      <c r="I31" t="str">
+        <v>2026-09-04T09:54:35.271Z</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>f738dccc-b7f4-4811-9f88-3e5ab1c3228e</v>
+      </c>
+      <c r="B32" t="str">
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+      </c>
+      <c r="C32" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="D32" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="E32" t="str">
+        <v>d2fa9872-abef-4790-bda1-7508469a2cd2</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Backlog</v>
+      </c>
+      <c r="G32" t="str">
+        <v>2026-09-04T09:54:48.369Z</v>
+      </c>
+      <c r="H32" t="str">
+        <v>2026-09-04T09:54:48.371Z</v>
+      </c>
+      <c r="I32" t="str">
+        <v>2026-09-04T09:54:48.371Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I32"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1048,16 +2847,223 @@
         <v>updatedAt</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>e5435e0d-9a20-4241-adc6-e880dc6bd3d2</v>
+      </c>
+      <c r="B2" t="str">
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+      </c>
+      <c r="C2" t="str">
+        <v>ผลตรวจสุขภาพ สัมพันธ์กับสรุปผลการตรวจสุขภาพ</v>
+      </c>
+      <c r="D2" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="E2" t="str">
+        <v>0</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-09-04T09:28:44.731Z</v>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-09-04T09:36:55.424Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>c9699cc1-1683-4feb-984e-878d32682885</v>
+      </c>
+      <c r="B3" t="str">
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+      </c>
+      <c r="C3" t="str">
+        <v>ผลการตรวจการตั้งครรภ์ ถ้าติ๊ก ตั้งครรภ์ ช่องผลการตรวจวัณโรคกับผลการตรวจโรคเท้าช้าง ให้เป็นทึบไปเลย เพราะไม่ได้มีการตรวจ</v>
+      </c>
+      <c r="D3" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="E3" t="str">
+        <v>1</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-09-04T09:28:53.342Z</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-09-04T09:36:55.440Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>4657d602-61e3-4999-8fd6-2b2eda534e20</v>
+      </c>
+      <c r="B4" t="str">
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+      </c>
+      <c r="C4" t="str">
+        <v>ส่วนใบรับรองแพทย์ ถ้า ผ่าน = สีเขียว, ประเภท 2 = สีเหลือง, ประเภท 3 = สีแดง</v>
+      </c>
+      <c r="D4" t="str">
+        <v>TRUE</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-09-04T09:29:00.544Z</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-09-04T09:36:56.844Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>47e9f838-dea2-451c-a4a6-7ad29c961c4a</v>
+      </c>
+      <c r="B5" t="str">
+        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Log ใบรับรองแพทย์ Collection ใหม่</v>
+      </c>
+      <c r="D5" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="E5" t="str">
+        <v>3</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-09-04T09:50:19.826Z</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-09-04T09:50:19.826Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>e7249296-600f-447c-9869-1d67655b3075</v>
+      </c>
+      <c r="B6" t="str">
+        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Log กรมธรรม์ไปใช้ Collection ใหม่</v>
+      </c>
+      <c r="D6" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="E6" t="str">
+        <v>4</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-09-04T09:50:30.949Z</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-09-04T09:50:30.949Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>b8311bf6-ddb0-4b10-9dae-f25584050fae</v>
+      </c>
+      <c r="B7" t="str">
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+      </c>
+      <c r="C7" t="str">
+        <v>เพิ่ม Log จัดการสิทธิ และแสดงข้อมูล</v>
+      </c>
+      <c r="D7" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="E7" t="str">
+        <v>5</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-09-04T09:51:24.363Z</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-09-04T09:51:24.363Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>168a98f3-0cdb-4081-8b06-92fc6a1b4f97</v>
+      </c>
+      <c r="B8" t="str">
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+      </c>
+      <c r="C8" t="str">
+        <v>เพิ่ม Log ลายเซ็น และแสดงข้อมูล</v>
+      </c>
+      <c r="D8" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="E8" t="str">
+        <v>6</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-09-04T09:51:30.264Z</v>
+      </c>
+      <c r="G8" t="str">
+        <v>2026-09-04T09:51:30.264Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>78826565-b6f0-4134-8ec5-51b689568502</v>
+      </c>
+      <c r="B9" t="str">
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+      </c>
+      <c r="C9" t="str">
+        <v>เพิ่ม Log ตั้งค่าระบบ และแสดงข้อมูล</v>
+      </c>
+      <c r="D9" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="E9" t="str">
+        <v>7</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-09-04T09:51:37.463Z</v>
+      </c>
+      <c r="G9" t="str">
+        <v>2026-09-04T09:51:37.463Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>d3abd120-8ba6-4dca-b36e-64c8291bcc93</v>
+      </c>
+      <c r="B10" t="str">
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+      </c>
+      <c r="C10" t="str">
+        <v>ปรับ Log Statement Collection ใหม่</v>
+      </c>
+      <c r="D10" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="E10" t="str">
+        <v>8</v>
+      </c>
+      <c r="F10" t="str">
+        <v>2026-09-04T09:51:43.481Z</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2026-09-04T09:51:43.481Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G10"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F30"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1079,9 +3085,589 @@
         <v>updatedAt</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ac8d7692-2e18-4474-b43d-1e1b085c3b72</v>
+      </c>
+      <c r="B2" t="str">
+        <v>a4db697d-4d50-4200-8355-647ab86cd480</v>
+      </c>
+      <c r="C2" t="str">
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+      </c>
+      <c r="D2" t="str">
+        <v>0</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-09-04T09:40:35.742Z</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-09-04T09:40:35.742Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>0f184845-2a39-46bf-84af-9f5d02bff128</v>
+      </c>
+      <c r="B3" t="str">
+        <v>62533ab0-8ef1-45b9-b2d4-961570759b92</v>
+      </c>
+      <c r="C3" t="str">
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+      </c>
+      <c r="D3" t="str">
+        <v>0</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-09-04T09:40:43.614Z</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-09-04T09:40:43.614Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>c13e3849-4301-4544-9fc0-32ab223dcf3a</v>
+      </c>
+      <c r="B4" t="str">
+        <v>62533ab0-8ef1-45b9-b2d4-961570759b92</v>
+      </c>
+      <c r="C4" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="D4" t="str">
+        <v>1</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-09-04T09:40:43.621Z</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-09-04T09:40:43.621Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>bc8a3094-100b-46c2-9ac1-d9b2d3582b5f</v>
+      </c>
+      <c r="B5" t="str">
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+      </c>
+      <c r="C5" t="str">
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+      </c>
+      <c r="D5" t="str">
+        <v>0</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-09-04T09:40:57.944Z</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-09-04T09:40:57.944Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>37e08404-2713-4dfe-936f-5f9322fa20e9</v>
+      </c>
+      <c r="B6" t="str">
+        <v>e0e2d398-49d2-4dc3-9fbc-512e2b97e4f5</v>
+      </c>
+      <c r="C6" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D6" t="str">
+        <v>0</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2026-09-04T09:41:08.413Z</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-09-04T09:41:08.413Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>c0934984-06c6-4ba5-9f45-c1b6e448bdbb</v>
+      </c>
+      <c r="B7" t="str">
+        <v>e0e2d398-49d2-4dc3-9fbc-512e2b97e4f5</v>
+      </c>
+      <c r="C7" t="str">
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+      </c>
+      <c r="D7" t="str">
+        <v>1</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2026-09-04T09:41:08.419Z</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-09-04T09:41:08.419Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>b81e12b4-20a5-4fc4-a514-50370afcac96</v>
+      </c>
+      <c r="B8" t="str">
+        <v>1e95dc95-6f63-4810-9d57-8520eb9b42c5</v>
+      </c>
+      <c r="C8" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D8" t="str">
+        <v>0</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2026-09-04T09:41:39.531Z</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-09-04T09:41:39.531Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>80990267-d989-453d-b6c0-934f6d17265e</v>
+      </c>
+      <c r="B9" t="str">
+        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
+      </c>
+      <c r="C9" t="str">
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+      </c>
+      <c r="D9" t="str">
+        <v>0</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2026-09-04T09:41:51.988Z</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-09-04T09:41:51.988Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>3f788bfd-4196-4334-b70e-e7d4f9aea927</v>
+      </c>
+      <c r="B10" t="str">
+        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
+      </c>
+      <c r="C10" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D10" t="str">
+        <v>1</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2026-09-04T09:41:51.994Z</v>
+      </c>
+      <c r="F10" t="str">
+        <v>2026-09-04T09:41:51.994Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>32c5e74c-e29b-49ce-8bb9-05c45ae2b05c</v>
+      </c>
+      <c r="B11" t="str">
+        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
+      </c>
+      <c r="C11" t="str">
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+      </c>
+      <c r="D11" t="str">
+        <v>0</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2026-09-04T09:42:00.043Z</v>
+      </c>
+      <c r="F11" t="str">
+        <v>2026-09-04T09:42:00.043Z</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>bc2310d5-a861-4446-b827-d5ca714102c1</v>
+      </c>
+      <c r="B12" t="str">
+        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
+      </c>
+      <c r="C12" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D12" t="str">
+        <v>1</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2026-09-04T09:42:00.049Z</v>
+      </c>
+      <c r="F12" t="str">
+        <v>2026-09-04T09:42:00.049Z</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>aa0c90a1-50a9-467e-aeff-a80e364d7231</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
+      </c>
+      <c r="C13" t="str">
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
+      </c>
+      <c r="D13" t="str">
+        <v>0</v>
+      </c>
+      <c r="E13" t="str">
+        <v>2026-09-04T09:42:08.465Z</v>
+      </c>
+      <c r="F13" t="str">
+        <v>2026-09-04T09:42:08.465Z</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>64fe364b-f395-498f-8813-6c1bba29fbc3</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
+      </c>
+      <c r="C14" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D14" t="str">
+        <v>1</v>
+      </c>
+      <c r="E14" t="str">
+        <v>2026-09-04T09:42:08.473Z</v>
+      </c>
+      <c r="F14" t="str">
+        <v>2026-09-04T09:42:08.473Z</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>1df7c234-174e-4ecc-86df-402763448af7</v>
+      </c>
+      <c r="B15" t="str">
+        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
+      </c>
+      <c r="C15" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="D15" t="str">
+        <v>0</v>
+      </c>
+      <c r="E15" t="str">
+        <v>2026-09-04T09:42:23.314Z</v>
+      </c>
+      <c r="F15" t="str">
+        <v>2026-09-04T09:42:23.314Z</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>2c5c97cc-6f06-4a34-b426-104fc1ef7003</v>
+      </c>
+      <c r="B16" t="str">
+        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
+      </c>
+      <c r="C16" t="str">
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+      </c>
+      <c r="D16" t="str">
+        <v>1</v>
+      </c>
+      <c r="E16" t="str">
+        <v>2026-09-04T09:42:23.320Z</v>
+      </c>
+      <c r="F16" t="str">
+        <v>2026-09-04T09:42:23.320Z</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>c2f765ad-b590-49db-b0a7-36e85e5895b4</v>
+      </c>
+      <c r="B17" t="str">
+        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
+      </c>
+      <c r="C17" t="str">
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+      </c>
+      <c r="D17" t="str">
+        <v>0</v>
+      </c>
+      <c r="E17" t="str">
+        <v>2026-09-04T09:42:32.095Z</v>
+      </c>
+      <c r="F17" t="str">
+        <v>2026-09-04T09:42:32.095Z</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>08a90228-bb97-418f-ac22-e80a3ba6b2cb</v>
+      </c>
+      <c r="B18" t="str">
+        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
+      </c>
+      <c r="C18" t="str">
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+      </c>
+      <c r="D18" t="str">
+        <v>1</v>
+      </c>
+      <c r="E18" t="str">
+        <v>2026-09-04T09:42:32.102Z</v>
+      </c>
+      <c r="F18" t="str">
+        <v>2026-09-04T09:42:32.102Z</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>9c12a7a8-f6ed-48d7-bd22-3b59c5cada75</v>
+      </c>
+      <c r="B19" t="str">
+        <v>d6acd7ea-e69f-4894-9ce4-c8ae86da6bd2</v>
+      </c>
+      <c r="C19" t="str">
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
+      </c>
+      <c r="D19" t="str">
+        <v>0</v>
+      </c>
+      <c r="E19" t="str">
+        <v>2026-09-04T09:42:39.367Z</v>
+      </c>
+      <c r="F19" t="str">
+        <v>2026-09-04T09:42:39.367Z</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>f8edc8fa-0fc6-44c4-a15c-14cfe4475d9e</v>
+      </c>
+      <c r="B20" t="str">
+        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
+      </c>
+      <c r="C20" t="str">
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+      </c>
+      <c r="D20" t="str">
+        <v>0</v>
+      </c>
+      <c r="E20" t="str">
+        <v>2026-09-04T09:44:49.319Z</v>
+      </c>
+      <c r="F20" t="str">
+        <v>2026-09-04T09:44:49.319Z</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>e1211e67-dde9-4873-a96f-6985e7753170</v>
+      </c>
+      <c r="B21" t="str">
+        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
+      </c>
+      <c r="C21" t="str">
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+      </c>
+      <c r="D21" t="str">
+        <v>1</v>
+      </c>
+      <c r="E21" t="str">
+        <v>2026-09-04T09:44:49.325Z</v>
+      </c>
+      <c r="F21" t="str">
+        <v>2026-09-04T09:44:49.325Z</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>5a79cab4-c5b3-4c96-8b5a-bf72005b39f2</v>
+      </c>
+      <c r="B22" t="str">
+        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
+      </c>
+      <c r="C22" t="str">
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+      </c>
+      <c r="D22" t="str">
+        <v>0</v>
+      </c>
+      <c r="E22" t="str">
+        <v>2026-09-04T09:45:22.504Z</v>
+      </c>
+      <c r="F22" t="str">
+        <v>2026-09-04T09:45:22.504Z</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>e16d77fc-e33d-4c73-be58-b8a0016c902a</v>
+      </c>
+      <c r="B23" t="str">
+        <v>12f8c884-7a9e-4086-8352-ace2ea778248</v>
+      </c>
+      <c r="C23" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="D23" t="str">
+        <v>0</v>
+      </c>
+      <c r="E23" t="str">
+        <v>2026-09-04T09:45:31.784Z</v>
+      </c>
+      <c r="F23" t="str">
+        <v>2026-09-04T09:45:31.784Z</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>76c55ffd-5c72-475c-9448-e969b036b7c0</v>
+      </c>
+      <c r="B24" t="str">
+        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
+      </c>
+      <c r="C24" t="str">
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+      </c>
+      <c r="D24" t="str">
+        <v>0</v>
+      </c>
+      <c r="E24" t="str">
+        <v>2026-09-04T09:47:39.835Z</v>
+      </c>
+      <c r="F24" t="str">
+        <v>2026-09-04T09:47:39.835Z</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>689f964d-b216-40de-881b-605919cf6b35</v>
+      </c>
+      <c r="B25" t="str">
+        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
+      </c>
+      <c r="C25" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D25" t="str">
+        <v>1</v>
+      </c>
+      <c r="E25" t="str">
+        <v>2026-09-04T09:47:39.839Z</v>
+      </c>
+      <c r="F25" t="str">
+        <v>2026-09-04T09:47:39.839Z</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>be30c4c5-9550-4b85-8401-c243a2cc9973</v>
+      </c>
+      <c r="B26" t="str">
+        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
+      </c>
+      <c r="C26" t="str">
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+      </c>
+      <c r="D26" t="str">
+        <v>0</v>
+      </c>
+      <c r="E26" t="str">
+        <v>2026-09-04T09:48:58.065Z</v>
+      </c>
+      <c r="F26" t="str">
+        <v>2026-09-04T09:48:58.065Z</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>6402d1cb-71a9-4249-9e8d-765a6d771490</v>
+      </c>
+      <c r="B27" t="str">
+        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
+      </c>
+      <c r="C27" t="str">
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+      </c>
+      <c r="D27" t="str">
+        <v>1</v>
+      </c>
+      <c r="E27" t="str">
+        <v>2026-09-04T09:48:58.069Z</v>
+      </c>
+      <c r="F27" t="str">
+        <v>2026-09-04T09:48:58.069Z</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>4aa09891-d7c9-447c-bfb3-f89253485b13</v>
+      </c>
+      <c r="B28" t="str">
+        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
+      </c>
+      <c r="C28" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="D28" t="str">
+        <v>0</v>
+      </c>
+      <c r="E28" t="str">
+        <v>2026-09-04T09:50:04.926Z</v>
+      </c>
+      <c r="F28" t="str">
+        <v>2026-09-04T09:50:04.926Z</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>deb50462-5b0f-499b-914d-68500cd93e57</v>
+      </c>
+      <c r="B29" t="str">
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+      </c>
+      <c r="C29" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="D29" t="str">
+        <v>0</v>
+      </c>
+      <c r="E29" t="str">
+        <v>2026-09-04T09:52:49.537Z</v>
+      </c>
+      <c r="F29" t="str">
+        <v>2026-09-04T09:52:49.537Z</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>4a562254-0467-4fdc-a082-c279f9803470</v>
+      </c>
+      <c r="B30" t="str">
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+      </c>
+      <c r="C30" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D30" t="str">
+        <v>1</v>
+      </c>
+      <c r="E30" t="str">
+        <v>2026-09-04T09:52:49.544Z</v>
+      </c>
+      <c r="F30" t="str">
+        <v>2026-09-04T09:52:49.544Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F30"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: enhance task and subtask management with assignee support
- Added `subtaskAssignments` model to the database schema for managing subtask assignees.
- Updated API endpoints to handle assignee IDs for subtasks during creation and updates.
- Enhanced task and subtask forms to support multiple assignees.
- Modified UI components to display and manage subtask assignees effectively.
- Updated Excel and Sheets repositories to include subtask assignee data.
</commit_message>
<xml_diff>
--- a/data/taskDB.xlsx
+++ b/data/taskDB.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Subtasks" sheetId="7" r:id="rId7"/>
     <sheet name="TaskAssignees" sheetId="8" r:id="rId8"/>
     <sheet name="TaskTypes" sheetId="9" r:id="rId9"/>
+    <sheet name="SubtaskAssignees" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -460,6 +461,237 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F11"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>subtaskId</v>
+      </c>
+      <c r="C1" t="str">
+        <v>teamMemberId</v>
+      </c>
+      <c r="D1" t="str">
+        <v>sortOrder</v>
+      </c>
+      <c r="E1" t="str">
+        <v>createdAt</v>
+      </c>
+      <c r="F1" t="str">
+        <v>updatedAt</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>cbc3ecad-b723-47f8-93ea-9d969a426285</v>
+      </c>
+      <c r="B2" t="str">
+        <v>e7249296-600f-447c-9869-1d67655b3075</v>
+      </c>
+      <c r="C2" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="D2" t="str">
+        <v>0</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-09-04T10:15:28.657Z</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-09-04T10:15:28.657Z</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>3735c245-12b7-4cda-8f14-5f0d3222faaa</v>
+      </c>
+      <c r="B3" t="str">
+        <v>47e9f838-dea2-451c-a4a6-7ad29c961c4a</v>
+      </c>
+      <c r="C3" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="D3" t="str">
+        <v>0</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-09-04T10:15:29.340Z</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-09-04T10:15:29.340Z</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>e83af4d7-838c-48b9-a9fa-f5244e739aa4</v>
+      </c>
+      <c r="B4" t="str">
+        <v>b8311bf6-ddb0-4b10-9dae-f25584050fae</v>
+      </c>
+      <c r="C4" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="D4" t="str">
+        <v>0</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-09-04T10:15:37.176Z</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-09-04T10:15:37.176Z</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>595e1a8b-ca2c-4fc8-804a-535b2f2dcae6</v>
+      </c>
+      <c r="B5" t="str">
+        <v>168a98f3-0cdb-4081-8b06-92fc6a1b4f97</v>
+      </c>
+      <c r="C5" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="D5" t="str">
+        <v>0</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-09-04T10:15:37.664Z</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-09-04T10:15:37.664Z</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>46d3ae73-749e-4864-98e4-e30149136b87</v>
+      </c>
+      <c r="B6" t="str">
+        <v>78826565-b6f0-4134-8ec5-51b689568502</v>
+      </c>
+      <c r="C6" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="D6" t="str">
+        <v>0</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2026-09-04T10:15:38.315Z</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-09-04T10:15:38.315Z</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>aa769b73-4795-45fd-99e0-3ba325ea9b83</v>
+      </c>
+      <c r="B7" t="str">
+        <v>d3abd120-8ba6-4dca-b36e-64c8291bcc93</v>
+      </c>
+      <c r="C7" t="str">
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+      </c>
+      <c r="D7" t="str">
+        <v>0</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2026-09-04T10:15:40.173Z</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-09-04T10:15:40.173Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>0f737fbb-ef65-448c-a0ce-84d90fe01c38</v>
+      </c>
+      <c r="B8" t="str">
+        <v>d3abd120-8ba6-4dca-b36e-64c8291bcc93</v>
+      </c>
+      <c r="C8" t="str">
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+      </c>
+      <c r="D8" t="str">
+        <v>1</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2026-09-04T10:15:40.180Z</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-09-04T10:15:40.180Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>d47d2637-7aee-4c15-9f28-7db15c5d735b</v>
+      </c>
+      <c r="B9" t="str">
+        <v>e5435e0d-9a20-4241-adc6-e880dc6bd3d2</v>
+      </c>
+      <c r="C9" t="str">
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+      </c>
+      <c r="D9" t="str">
+        <v>0</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2026-09-04T10:15:49.861Z</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-09-04T10:15:49.861Z</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>888a6d5c-c169-4644-ad30-0aa6b9d3048a</v>
+      </c>
+      <c r="B10" t="str">
+        <v>c9699cc1-1683-4feb-984e-878d32682885</v>
+      </c>
+      <c r="C10" t="str">
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+      </c>
+      <c r="D10" t="str">
+        <v>0</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2026-09-04T10:15:50.569Z</v>
+      </c>
+      <c r="F10" t="str">
+        <v>2026-09-04T10:15:50.569Z</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>1a7cd58c-3775-46bf-8b3b-0793b1e36035</v>
+      </c>
+      <c r="B11" t="str">
+        <v>4657d602-61e3-4999-8fd6-2b2eda534e20</v>
+      </c>
+      <c r="C11" t="str">
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+      </c>
+      <c r="D11" t="str">
+        <v>0</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2026-09-04T10:15:51.162Z</v>
+      </c>
+      <c r="F11" t="str">
+        <v>2026-09-04T10:15:51.162Z</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
@@ -1271,7 +1503,7 @@
         <v>2026-09-04T09:27:00.612Z</v>
       </c>
       <c r="P7" t="str">
-        <v>2026-09-04T09:40:57.950Z</v>
+        <v>2026-09-04T10:15:52.853Z</v>
       </c>
     </row>
     <row r="8">
@@ -1821,7 +2053,7 @@
         <v>2026-09-04T09:50:04.917Z</v>
       </c>
       <c r="P18" t="str">
-        <v>2026-09-04T09:50:04.931Z</v>
+        <v>2026-09-04T10:15:31.436Z</v>
       </c>
     </row>
     <row r="19">
@@ -1871,7 +2103,7 @@
         <v>2026-09-04T09:51:03.522Z</v>
       </c>
       <c r="P19" t="str">
-        <v>2026-09-04T09:54:48.379Z</v>
+        <v>2026-09-04T10:15:41.981Z</v>
       </c>
     </row>
   </sheetData>
@@ -2867,7 +3099,7 @@
         <v>2026-09-04T09:28:44.731Z</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-09-04T09:36:55.424Z</v>
+        <v>2026-09-04T10:15:49.842Z</v>
       </c>
     </row>
     <row r="3">
@@ -2890,7 +3122,7 @@
         <v>2026-09-04T09:28:53.342Z</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-09-04T09:36:55.440Z</v>
+        <v>2026-09-04T10:15:50.555Z</v>
       </c>
     </row>
     <row r="4">
@@ -2913,7 +3145,7 @@
         <v>2026-09-04T09:29:00.544Z</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-09-04T09:36:56.844Z</v>
+        <v>2026-09-04T10:15:51.145Z</v>
       </c>
     </row>
     <row r="5">
@@ -2936,7 +3168,7 @@
         <v>2026-09-04T09:50:19.826Z</v>
       </c>
       <c r="G5" t="str">
-        <v>2026-09-04T09:50:19.826Z</v>
+        <v>2026-09-04T10:15:29.325Z</v>
       </c>
     </row>
     <row r="6">
@@ -2959,7 +3191,7 @@
         <v>2026-09-04T09:50:30.949Z</v>
       </c>
       <c r="G6" t="str">
-        <v>2026-09-04T09:50:30.949Z</v>
+        <v>2026-09-04T10:15:28.638Z</v>
       </c>
     </row>
     <row r="7">
@@ -2982,7 +3214,7 @@
         <v>2026-09-04T09:51:24.363Z</v>
       </c>
       <c r="G7" t="str">
-        <v>2026-09-04T09:51:24.363Z</v>
+        <v>2026-09-04T10:15:37.156Z</v>
       </c>
     </row>
     <row r="8">
@@ -3005,7 +3237,7 @@
         <v>2026-09-04T09:51:30.264Z</v>
       </c>
       <c r="G8" t="str">
-        <v>2026-09-04T09:51:30.264Z</v>
+        <v>2026-09-04T10:15:37.653Z</v>
       </c>
     </row>
     <row r="9">
@@ -3028,7 +3260,7 @@
         <v>2026-09-04T09:51:37.463Z</v>
       </c>
       <c r="G9" t="str">
-        <v>2026-09-04T09:51:37.463Z</v>
+        <v>2026-09-04T10:15:38.297Z</v>
       </c>
     </row>
     <row r="10">
@@ -3051,7 +3283,7 @@
         <v>2026-09-04T09:51:43.481Z</v>
       </c>
       <c r="G10" t="str">
-        <v>2026-09-04T09:51:43.481Z</v>
+        <v>2026-09-04T10:15:40.154Z</v>
       </c>
     </row>
   </sheetData>
@@ -3147,470 +3379,470 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>bc8a3094-100b-46c2-9ac1-d9b2d3582b5f</v>
+        <v>37e08404-2713-4dfe-936f-5f9322fa20e9</v>
       </c>
       <c r="B5" t="str">
-        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+        <v>e0e2d398-49d2-4dc3-9fbc-512e2b97e4f5</v>
       </c>
       <c r="C5" t="str">
-        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D5" t="str">
         <v>0</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-09-04T09:40:57.944Z</v>
+        <v>2026-09-04T09:41:08.413Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-04T09:40:57.944Z</v>
+        <v>2026-09-04T09:41:08.413Z</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>37e08404-2713-4dfe-936f-5f9322fa20e9</v>
+        <v>c0934984-06c6-4ba5-9f45-c1b6e448bdbb</v>
       </c>
       <c r="B6" t="str">
         <v>e0e2d398-49d2-4dc3-9fbc-512e2b97e4f5</v>
       </c>
       <c r="C6" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="D6" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="str">
-        <v>2026-09-04T09:41:08.413Z</v>
+        <v>2026-09-04T09:41:08.419Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-04T09:41:08.413Z</v>
+        <v>2026-09-04T09:41:08.419Z</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>c0934984-06c6-4ba5-9f45-c1b6e448bdbb</v>
+        <v>b81e12b4-20a5-4fc4-a514-50370afcac96</v>
       </c>
       <c r="B7" t="str">
-        <v>e0e2d398-49d2-4dc3-9fbc-512e2b97e4f5</v>
+        <v>1e95dc95-6f63-4810-9d57-8520eb9b42c5</v>
       </c>
       <c r="C7" t="str">
-        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D7" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-09-04T09:41:08.419Z</v>
+        <v>2026-09-04T09:41:39.531Z</v>
       </c>
       <c r="F7" t="str">
-        <v>2026-09-04T09:41:08.419Z</v>
+        <v>2026-09-04T09:41:39.531Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>b81e12b4-20a5-4fc4-a514-50370afcac96</v>
+        <v>80990267-d989-453d-b6c0-934f6d17265e</v>
       </c>
       <c r="B8" t="str">
-        <v>1e95dc95-6f63-4810-9d57-8520eb9b42c5</v>
+        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
       </c>
       <c r="C8" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D8" t="str">
         <v>0</v>
       </c>
       <c r="E8" t="str">
-        <v>2026-09-04T09:41:39.531Z</v>
+        <v>2026-09-04T09:41:51.988Z</v>
       </c>
       <c r="F8" t="str">
-        <v>2026-09-04T09:41:39.531Z</v>
+        <v>2026-09-04T09:41:51.988Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>80990267-d989-453d-b6c0-934f6d17265e</v>
+        <v>3f788bfd-4196-4334-b70e-e7d4f9aea927</v>
       </c>
       <c r="B9" t="str">
         <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
       </c>
       <c r="C9" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D9" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="str">
-        <v>2026-09-04T09:41:51.988Z</v>
+        <v>2026-09-04T09:41:51.994Z</v>
       </c>
       <c r="F9" t="str">
-        <v>2026-09-04T09:41:51.988Z</v>
+        <v>2026-09-04T09:41:51.994Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>3f788bfd-4196-4334-b70e-e7d4f9aea927</v>
+        <v>32c5e74c-e29b-49ce-8bb9-05c45ae2b05c</v>
       </c>
       <c r="B10" t="str">
-        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
+        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
       </c>
       <c r="C10" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D10" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" t="str">
-        <v>2026-09-04T09:41:51.994Z</v>
+        <v>2026-09-04T09:42:00.043Z</v>
       </c>
       <c r="F10" t="str">
-        <v>2026-09-04T09:41:51.994Z</v>
+        <v>2026-09-04T09:42:00.043Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>32c5e74c-e29b-49ce-8bb9-05c45ae2b05c</v>
+        <v>bc2310d5-a861-4446-b827-d5ca714102c1</v>
       </c>
       <c r="B11" t="str">
         <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
       </c>
       <c r="C11" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D11" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" t="str">
-        <v>2026-09-04T09:42:00.043Z</v>
+        <v>2026-09-04T09:42:00.049Z</v>
       </c>
       <c r="F11" t="str">
-        <v>2026-09-04T09:42:00.043Z</v>
+        <v>2026-09-04T09:42:00.049Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>bc2310d5-a861-4446-b827-d5ca714102c1</v>
+        <v>aa0c90a1-50a9-467e-aeff-a80e364d7231</v>
       </c>
       <c r="B12" t="str">
-        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
+        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
       </c>
       <c r="C12" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
       <c r="D12" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" t="str">
-        <v>2026-09-04T09:42:00.049Z</v>
+        <v>2026-09-04T09:42:08.465Z</v>
       </c>
       <c r="F12" t="str">
-        <v>2026-09-04T09:42:00.049Z</v>
+        <v>2026-09-04T09:42:08.465Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>aa0c90a1-50a9-467e-aeff-a80e364d7231</v>
+        <v>64fe364b-f395-498f-8813-6c1bba29fbc3</v>
       </c>
       <c r="B13" t="str">
         <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
       </c>
       <c r="C13" t="str">
-        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D13" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" t="str">
-        <v>2026-09-04T09:42:08.465Z</v>
+        <v>2026-09-04T09:42:08.473Z</v>
       </c>
       <c r="F13" t="str">
-        <v>2026-09-04T09:42:08.465Z</v>
+        <v>2026-09-04T09:42:08.473Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>64fe364b-f395-498f-8813-6c1bba29fbc3</v>
+        <v>1df7c234-174e-4ecc-86df-402763448af7</v>
       </c>
       <c r="B14" t="str">
-        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
+        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
       </c>
       <c r="C14" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="D14" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" t="str">
-        <v>2026-09-04T09:42:08.473Z</v>
+        <v>2026-09-04T09:42:23.314Z</v>
       </c>
       <c r="F14" t="str">
-        <v>2026-09-04T09:42:08.473Z</v>
+        <v>2026-09-04T09:42:23.314Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>1df7c234-174e-4ecc-86df-402763448af7</v>
+        <v>2c5c97cc-6f06-4a34-b426-104fc1ef7003</v>
       </c>
       <c r="B15" t="str">
         <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
       </c>
       <c r="C15" t="str">
-        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D15" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="str">
-        <v>2026-09-04T09:42:23.314Z</v>
+        <v>2026-09-04T09:42:23.320Z</v>
       </c>
       <c r="F15" t="str">
-        <v>2026-09-04T09:42:23.314Z</v>
+        <v>2026-09-04T09:42:23.320Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2c5c97cc-6f06-4a34-b426-104fc1ef7003</v>
+        <v>c2f765ad-b590-49db-b0a7-36e85e5895b4</v>
       </c>
       <c r="B16" t="str">
-        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
+        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
       </c>
       <c r="C16" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="D16" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" t="str">
-        <v>2026-09-04T09:42:23.320Z</v>
+        <v>2026-09-04T09:42:32.095Z</v>
       </c>
       <c r="F16" t="str">
-        <v>2026-09-04T09:42:23.320Z</v>
+        <v>2026-09-04T09:42:32.095Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>c2f765ad-b590-49db-b0a7-36e85e5895b4</v>
+        <v>08a90228-bb97-418f-ac22-e80a3ba6b2cb</v>
       </c>
       <c r="B17" t="str">
         <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
       </c>
       <c r="C17" t="str">
-        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D17" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" t="str">
-        <v>2026-09-04T09:42:32.095Z</v>
+        <v>2026-09-04T09:42:32.102Z</v>
       </c>
       <c r="F17" t="str">
-        <v>2026-09-04T09:42:32.095Z</v>
+        <v>2026-09-04T09:42:32.102Z</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>08a90228-bb97-418f-ac22-e80a3ba6b2cb</v>
+        <v>9c12a7a8-f6ed-48d7-bd22-3b59c5cada75</v>
       </c>
       <c r="B18" t="str">
-        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
+        <v>d6acd7ea-e69f-4894-9ce4-c8ae86da6bd2</v>
       </c>
       <c r="C18" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
       <c r="D18" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E18" t="str">
-        <v>2026-09-04T09:42:32.102Z</v>
+        <v>2026-09-04T09:42:39.367Z</v>
       </c>
       <c r="F18" t="str">
-        <v>2026-09-04T09:42:32.102Z</v>
+        <v>2026-09-04T09:42:39.367Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>9c12a7a8-f6ed-48d7-bd22-3b59c5cada75</v>
+        <v>f8edc8fa-0fc6-44c4-a15c-14cfe4475d9e</v>
       </c>
       <c r="B19" t="str">
-        <v>d6acd7ea-e69f-4894-9ce4-c8ae86da6bd2</v>
+        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
       </c>
       <c r="C19" t="str">
-        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D19" t="str">
         <v>0</v>
       </c>
       <c r="E19" t="str">
-        <v>2026-09-04T09:42:39.367Z</v>
+        <v>2026-09-04T09:44:49.319Z</v>
       </c>
       <c r="F19" t="str">
-        <v>2026-09-04T09:42:39.367Z</v>
+        <v>2026-09-04T09:44:49.319Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>f8edc8fa-0fc6-44c4-a15c-14cfe4475d9e</v>
+        <v>e1211e67-dde9-4873-a96f-6985e7753170</v>
       </c>
       <c r="B20" t="str">
         <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
       </c>
       <c r="C20" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D20" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E20" t="str">
-        <v>2026-09-04T09:44:49.319Z</v>
+        <v>2026-09-04T09:44:49.325Z</v>
       </c>
       <c r="F20" t="str">
-        <v>2026-09-04T09:44:49.319Z</v>
+        <v>2026-09-04T09:44:49.325Z</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>e1211e67-dde9-4873-a96f-6985e7753170</v>
+        <v>5a79cab4-c5b3-4c96-8b5a-bf72005b39f2</v>
       </c>
       <c r="B21" t="str">
-        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
+        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
       </c>
       <c r="C21" t="str">
         <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D21" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21" t="str">
-        <v>2026-09-04T09:44:49.325Z</v>
+        <v>2026-09-04T09:45:22.504Z</v>
       </c>
       <c r="F21" t="str">
-        <v>2026-09-04T09:44:49.325Z</v>
+        <v>2026-09-04T09:45:22.504Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>5a79cab4-c5b3-4c96-8b5a-bf72005b39f2</v>
+        <v>e16d77fc-e33d-4c73-be58-b8a0016c902a</v>
       </c>
       <c r="B22" t="str">
-        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
+        <v>12f8c884-7a9e-4086-8352-ace2ea778248</v>
       </c>
       <c r="C22" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="D22" t="str">
         <v>0</v>
       </c>
       <c r="E22" t="str">
-        <v>2026-09-04T09:45:22.504Z</v>
+        <v>2026-09-04T09:45:31.784Z</v>
       </c>
       <c r="F22" t="str">
-        <v>2026-09-04T09:45:22.504Z</v>
+        <v>2026-09-04T09:45:31.784Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>e16d77fc-e33d-4c73-be58-b8a0016c902a</v>
+        <v>76c55ffd-5c72-475c-9448-e969b036b7c0</v>
       </c>
       <c r="B23" t="str">
-        <v>12f8c884-7a9e-4086-8352-ace2ea778248</v>
+        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
       </c>
       <c r="C23" t="str">
-        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D23" t="str">
         <v>0</v>
       </c>
       <c r="E23" t="str">
-        <v>2026-09-04T09:45:31.784Z</v>
+        <v>2026-09-04T09:47:39.835Z</v>
       </c>
       <c r="F23" t="str">
-        <v>2026-09-04T09:45:31.784Z</v>
+        <v>2026-09-04T09:47:39.835Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>76c55ffd-5c72-475c-9448-e969b036b7c0</v>
+        <v>689f964d-b216-40de-881b-605919cf6b35</v>
       </c>
       <c r="B24" t="str">
         <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
       </c>
       <c r="C24" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D24" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" t="str">
-        <v>2026-09-04T09:47:39.835Z</v>
+        <v>2026-09-04T09:47:39.839Z</v>
       </c>
       <c r="F24" t="str">
-        <v>2026-09-04T09:47:39.835Z</v>
+        <v>2026-09-04T09:47:39.839Z</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>689f964d-b216-40de-881b-605919cf6b35</v>
+        <v>be30c4c5-9550-4b85-8401-c243a2cc9973</v>
       </c>
       <c r="B25" t="str">
-        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
+        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
       </c>
       <c r="C25" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D25" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" t="str">
-        <v>2026-09-04T09:47:39.839Z</v>
+        <v>2026-09-04T09:48:58.065Z</v>
       </c>
       <c r="F25" t="str">
-        <v>2026-09-04T09:47:39.839Z</v>
+        <v>2026-09-04T09:48:58.065Z</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>be30c4c5-9550-4b85-8401-c243a2cc9973</v>
+        <v>6402d1cb-71a9-4249-9e8d-765a6d771490</v>
       </c>
       <c r="B26" t="str">
         <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
       </c>
       <c r="C26" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D26" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E26" t="str">
-        <v>2026-09-04T09:48:58.065Z</v>
+        <v>2026-09-04T09:48:58.069Z</v>
       </c>
       <c r="F26" t="str">
-        <v>2026-09-04T09:48:58.065Z</v>
+        <v>2026-09-04T09:48:58.069Z</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>6402d1cb-71a9-4249-9e8d-765a6d771490</v>
+        <v>837b7f6d-8aa7-4477-a101-2bc781f457eb</v>
       </c>
       <c r="B27" t="str">
-        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
+        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
       </c>
       <c r="C27" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="D27" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" t="str">
-        <v>2026-09-04T09:48:58.069Z</v>
+        <v>2026-09-04T10:15:31.431Z</v>
       </c>
       <c r="F27" t="str">
-        <v>2026-09-04T09:48:58.069Z</v>
+        <v>2026-09-04T10:15:31.431Z</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>4aa09891-d7c9-447c-bfb3-f89253485b13</v>
+        <v>eb5d9e38-bcca-4ed1-93e8-a4d8d83273e3</v>
       </c>
       <c r="B28" t="str">
-        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
       </c>
       <c r="C28" t="str">
         <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
@@ -3619,50 +3851,50 @@
         <v>0</v>
       </c>
       <c r="E28" t="str">
-        <v>2026-09-04T09:50:04.926Z</v>
+        <v>2026-09-04T10:15:41.968Z</v>
       </c>
       <c r="F28" t="str">
-        <v>2026-09-04T09:50:04.926Z</v>
+        <v>2026-09-04T10:15:41.968Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>deb50462-5b0f-499b-914d-68500cd93e57</v>
+        <v>c9ac57b0-fc08-4608-b8dd-07c6f31fd162</v>
       </c>
       <c r="B29" t="str">
         <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
       </c>
       <c r="C29" t="str">
-        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D29" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" t="str">
-        <v>2026-09-04T09:52:49.537Z</v>
+        <v>2026-09-04T10:15:41.975Z</v>
       </c>
       <c r="F29" t="str">
-        <v>2026-09-04T09:52:49.537Z</v>
+        <v>2026-09-04T10:15:41.975Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>4a562254-0467-4fdc-a082-c279f9803470</v>
+        <v>7bac2115-77f1-401f-ba0e-824e6d60f4fd</v>
       </c>
       <c r="B30" t="str">
-        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
       </c>
       <c r="C30" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="D30" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E30" t="str">
-        <v>2026-09-04T09:52:49.544Z</v>
+        <v>2026-09-04T10:15:52.847Z</v>
       </c>
       <c r="F30" t="str">
-        <v>2026-09-04T09:52:49.544Z</v>
+        <v>2026-09-04T10:15:52.847Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: enhance task management with inline assignee editing and calendar view improvements
- Added inline editing for team member assignments in the task list view.
- Introduced a new `InlineAssigneePicker` component for better assignee management.
- Updated task calendar view to display UAT and PRD timelines with visual indicators.
- Refactored task filtering logic to show tasks based on specific dates.
- Enhanced settings dialog to support editing team member details.
</commit_message>
<xml_diff>
--- a/data/taskDB.xlsx
+++ b/data/taskDB.xlsx
@@ -463,7 +463,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -587,50 +587,50 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>aa769b73-4795-45fd-99e0-3ba325ea9b83</v>
+        <v>d47d2637-7aee-4c15-9f28-7db15c5d735b</v>
       </c>
       <c r="B7" t="str">
-        <v>d3abd120-8ba6-4dca-b36e-64c8291bcc93</v>
+        <v>e5435e0d-9a20-4241-adc6-e880dc6bd3d2</v>
       </c>
       <c r="C7" t="str">
-        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="D7" t="str">
         <v>0</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-09-04T10:15:40.173Z</v>
+        <v>2026-09-04T10:15:49.861Z</v>
       </c>
       <c r="F7" t="str">
-        <v>2026-09-04T10:15:40.173Z</v>
+        <v>2026-09-04T10:15:49.861Z</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>0f737fbb-ef65-448c-a0ce-84d90fe01c38</v>
+        <v>888a6d5c-c169-4644-ad30-0aa6b9d3048a</v>
       </c>
       <c r="B8" t="str">
-        <v>d3abd120-8ba6-4dca-b36e-64c8291bcc93</v>
+        <v>c9699cc1-1683-4feb-984e-878d32682885</v>
       </c>
       <c r="C8" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="D8" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" t="str">
-        <v>2026-09-04T10:15:40.180Z</v>
+        <v>2026-09-04T10:15:50.569Z</v>
       </c>
       <c r="F8" t="str">
-        <v>2026-09-04T10:15:40.180Z</v>
+        <v>2026-09-04T10:15:50.569Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>d47d2637-7aee-4c15-9f28-7db15c5d735b</v>
+        <v>1a7cd58c-3775-46bf-8b3b-0793b1e36035</v>
       </c>
       <c r="B9" t="str">
-        <v>e5435e0d-9a20-4241-adc6-e880dc6bd3d2</v>
+        <v>4657d602-61e3-4999-8fd6-2b2eda534e20</v>
       </c>
       <c r="C9" t="str">
         <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
@@ -639,55 +639,35 @@
         <v>0</v>
       </c>
       <c r="E9" t="str">
-        <v>2026-09-04T10:15:49.861Z</v>
+        <v>2026-09-04T10:15:51.162Z</v>
       </c>
       <c r="F9" t="str">
-        <v>2026-09-04T10:15:49.861Z</v>
+        <v>2026-09-04T10:15:51.162Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>888a6d5c-c169-4644-ad30-0aa6b9d3048a</v>
+        <v>3f02a3c6-4846-489a-8ad3-8add2bd12235</v>
       </c>
       <c r="B10" t="str">
-        <v>c9699cc1-1683-4feb-984e-878d32682885</v>
+        <v>d3abd120-8ba6-4dca-b36e-64c8291bcc93</v>
       </c>
       <c r="C10" t="str">
-        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D10" t="str">
         <v>0</v>
       </c>
       <c r="E10" t="str">
-        <v>2026-09-04T10:15:50.569Z</v>
+        <v>2026-09-04T11:41:47.465Z</v>
       </c>
       <c r="F10" t="str">
-        <v>2026-09-04T10:15:50.569Z</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>1a7cd58c-3775-46bf-8b3b-0793b1e36035</v>
-      </c>
-      <c r="B11" t="str">
-        <v>4657d602-61e3-4999-8fd6-2b2eda534e20</v>
-      </c>
-      <c r="C11" t="str">
-        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
-      </c>
-      <c r="D11" t="str">
-        <v>0</v>
-      </c>
-      <c r="E11" t="str">
-        <v>2026-09-04T10:15:51.162Z</v>
-      </c>
-      <c r="F11" t="str">
-        <v>2026-09-04T10:15:51.162Z</v>
+        <v>2026-09-04T11:41:47.465Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -785,7 +765,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -858,13 +838,13 @@
         <v>#22C55E</v>
       </c>
       <c r="D4" t="str">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E4" t="str">
         <v>2026-09-01T07:23:24.983Z</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-09-04T08:58:01.424Z</v>
+        <v>2026-09-04T11:33:02.517Z</v>
       </c>
     </row>
     <row r="5">
@@ -878,13 +858,13 @@
         <v>#F97316</v>
       </c>
       <c r="D5" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5" t="str">
         <v>2026-09-01T07:23:24.985Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-04T08:58:01.421Z</v>
+        <v>2026-09-04T11:33:02.520Z</v>
       </c>
     </row>
     <row r="6">
@@ -898,38 +878,18 @@
         <v>#6BB82A</v>
       </c>
       <c r="D6" t="str">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E6" t="str">
         <v>2026-09-01T07:23:24.988Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-04T08:58:01.419Z</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>0ba0e5b4-b8f1-47b6-ab62-754441e3810d</v>
-      </c>
-      <c r="B7" t="str">
-        <v>TEST</v>
-      </c>
-      <c r="C7" t="str">
-        <v>#EC4899</v>
-      </c>
-      <c r="D7" t="str">
-        <v>4</v>
-      </c>
-      <c r="E7" t="str">
-        <v>2026-09-04T07:23:00.313Z</v>
-      </c>
-      <c r="F7" t="str">
-        <v>2026-09-04T07:27:11.498Z</v>
+        <v>2026-09-04T11:33:02.514Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -966,7 +926,7 @@
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="B2" t="str">
-        <v>กัน</v>
+        <v>Guny</v>
       </c>
       <c r="C2" t="str">
         <v>#22C55E</v>
@@ -981,7 +941,7 @@
         <v>2026-09-01T07:26:41.854Z</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-09-01T07:26:41.854Z</v>
+        <v>2026-09-04T11:53:20.413Z</v>
       </c>
     </row>
     <row r="3">
@@ -989,7 +949,7 @@
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="B3" t="str">
-        <v>ครีม</v>
+        <v>Cream</v>
       </c>
       <c r="C3" t="str">
         <v>#EF4444</v>
@@ -1004,7 +964,7 @@
         <v>2026-09-04T08:31:09.214Z</v>
       </c>
       <c r="G3" t="str">
-        <v>2026-09-04T08:31:09.214Z</v>
+        <v>2026-09-04T11:53:27.762Z</v>
       </c>
     </row>
     <row r="4">
@@ -1012,7 +972,7 @@
         <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="B4" t="str">
-        <v>พี่เอก</v>
+        <v>P Aek</v>
       </c>
       <c r="C4" t="str">
         <v>#F97316</v>
@@ -1027,7 +987,7 @@
         <v>2026-09-04T08:31:15.973Z</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-09-04T08:31:15.973Z</v>
+        <v>2026-09-04T11:53:35.476Z</v>
       </c>
     </row>
     <row r="5">
@@ -1035,7 +995,7 @@
         <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="B5" t="str">
-        <v>พี่จู</v>
+        <v>P Juu</v>
       </c>
       <c r="C5" t="str">
         <v>#3B82F6</v>
@@ -1050,7 +1010,7 @@
         <v>2026-09-04T08:31:24.760Z</v>
       </c>
       <c r="G5" t="str">
-        <v>2026-09-04T08:31:24.760Z</v>
+        <v>2026-09-04T11:53:44.607Z</v>
       </c>
     </row>
     <row r="6">
@@ -1058,7 +1018,7 @@
         <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
       <c r="B6" t="str">
-        <v>ตาเฟม</v>
+        <v>Frame</v>
       </c>
       <c r="C6" t="str">
         <v>#8B5CF6</v>
@@ -1073,7 +1033,7 @@
         <v>2026-09-04T08:31:29.670Z</v>
       </c>
       <c r="G6" t="str">
-        <v>2026-09-04T08:31:29.670Z</v>
+        <v>2026-09-04T11:53:59.480Z</v>
       </c>
     </row>
     <row r="7">
@@ -1081,7 +1041,7 @@
         <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="B7" t="str">
-        <v>มาย</v>
+        <v>Mild</v>
       </c>
       <c r="C7" t="str">
         <v>#EC4899</v>
@@ -1096,7 +1056,7 @@
         <v>2026-09-04T08:31:33.588Z</v>
       </c>
       <c r="G7" t="str">
-        <v>2026-09-04T08:31:33.588Z</v>
+        <v>2026-09-04T11:54:13.639Z</v>
       </c>
     </row>
     <row r="8">
@@ -1104,7 +1064,7 @@
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="B8" t="str">
-        <v>บรีส</v>
+        <v>Breez</v>
       </c>
       <c r="C8" t="str">
         <v>#75D7F0</v>
@@ -1119,7 +1079,7 @@
         <v>2026-09-04T08:31:52.262Z</v>
       </c>
       <c r="G8" t="str">
-        <v>2026-09-04T08:31:52.262Z</v>
+        <v>2026-09-04T11:54:20.446Z</v>
       </c>
     </row>
     <row r="9">
@@ -1127,7 +1087,7 @@
         <v>190c2d73-d236-4277-a3e1-b6004555ac94</v>
       </c>
       <c r="B9" t="str">
-        <v>พริ้ง</v>
+        <v>Prink</v>
       </c>
       <c r="C9" t="str">
         <v>#F0EC75</v>
@@ -1142,7 +1102,7 @@
         <v>2026-09-04T08:32:04.538Z</v>
       </c>
       <c r="G9" t="str">
-        <v>2026-09-04T08:32:04.538Z</v>
+        <v>2026-09-04T11:54:26.641Z</v>
       </c>
     </row>
   </sheetData>
@@ -1494,7 +1454,7 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M7" t="str">
-        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
       <c r="N7" t="str">
         <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
@@ -1503,7 +1463,7 @@
         <v>2026-09-04T09:27:00.612Z</v>
       </c>
       <c r="P7" t="str">
-        <v>2026-09-04T10:15:52.853Z</v>
+        <v>2026-09-04T11:32:30.909Z</v>
       </c>
     </row>
     <row r="8">
@@ -1644,7 +1604,7 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M10" t="str">
-        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
       </c>
       <c r="N10" t="str">
         <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
@@ -1653,7 +1613,7 @@
         <v>2026-09-04T09:33:03.132Z</v>
       </c>
       <c r="P10" t="str">
-        <v>2026-09-04T09:40:43.627Z</v>
+        <v>2026-09-04T11:32:35.144Z</v>
       </c>
     </row>
     <row r="11">
@@ -2103,7 +2063,7 @@
         <v>2026-09-04T09:51:03.522Z</v>
       </c>
       <c r="P19" t="str">
-        <v>2026-09-04T10:15:41.981Z</v>
+        <v>2026-09-04T11:41:49.865Z</v>
       </c>
     </row>
   </sheetData>
@@ -2115,7 +2075,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I34"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3045,9 +3005,67 @@
         <v>2026-09-04T09:54:48.371Z</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>95a80a71-da67-45b4-bad8-36f2327f34e8</v>
+      </c>
+      <c r="B33" t="str">
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+      </c>
+      <c r="C33" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="D33" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="E33" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="F33" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="G33" t="str">
+        <v>2026-09-04T11:32:30.898Z</v>
+      </c>
+      <c r="H33" t="str">
+        <v>2026-09-04T11:32:30.900Z</v>
+      </c>
+      <c r="I33" t="str">
+        <v>2026-09-04T11:32:30.900Z</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>aa434cc2-baf0-4ef6-a826-9555d2fdc29a</v>
+      </c>
+      <c r="B34" t="str">
+        <v>62533ab0-8ef1-45b9-b2d4-961570759b92</v>
+      </c>
+      <c r="C34" t="str">
+        <v>45382819-dfd5-4193-99a0-dd906551cce0</v>
+      </c>
+      <c r="D34" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="E34" t="str">
+        <v>9f787cec-a7e0-4b6a-9319-8e90c5189911</v>
+      </c>
+      <c r="F34" t="str">
+        <v>UAT</v>
+      </c>
+      <c r="G34" t="str">
+        <v>2026-09-04T11:32:35.133Z</v>
+      </c>
+      <c r="H34" t="str">
+        <v>2026-09-04T11:32:35.136Z</v>
+      </c>
+      <c r="I34" t="str">
+        <v>2026-09-04T11:32:35.136Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I34"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3283,7 +3301,7 @@
         <v>2026-09-04T09:51:43.481Z</v>
       </c>
       <c r="G10" t="str">
-        <v>2026-09-04T10:15:40.154Z</v>
+        <v>2026-09-04T11:41:47.445Z</v>
       </c>
     </row>
   </sheetData>
@@ -3839,62 +3857,62 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>eb5d9e38-bcca-4ed1-93e8-a4d8d83273e3</v>
+        <v>7bac2115-77f1-401f-ba0e-824e6d60f4fd</v>
       </c>
       <c r="B28" t="str">
-        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
       </c>
       <c r="C28" t="str">
-        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="D28" t="str">
         <v>0</v>
       </c>
       <c r="E28" t="str">
-        <v>2026-09-04T10:15:41.968Z</v>
+        <v>2026-09-04T10:15:52.847Z</v>
       </c>
       <c r="F28" t="str">
-        <v>2026-09-04T10:15:41.968Z</v>
+        <v>2026-09-04T10:15:52.847Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>c9ac57b0-fc08-4608-b8dd-07c6f31fd162</v>
+        <v>4e27d0ea-d725-4fd6-8af3-af70d286f196</v>
       </c>
       <c r="B29" t="str">
         <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
       </c>
       <c r="C29" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="D29" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E29" t="str">
-        <v>2026-09-04T10:15:41.975Z</v>
+        <v>2026-09-04T11:41:49.851Z</v>
       </c>
       <c r="F29" t="str">
-        <v>2026-09-04T10:15:41.975Z</v>
+        <v>2026-09-04T11:41:49.851Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>7bac2115-77f1-401f-ba0e-824e6d60f4fd</v>
+        <v>9c21d982-7ad7-4a32-8875-f8af532fdf47</v>
       </c>
       <c r="B30" t="str">
-        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
       </c>
       <c r="C30" t="str">
-        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D30" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E30" t="str">
-        <v>2026-09-04T10:15:52.847Z</v>
+        <v>2026-09-04T11:41:49.858Z</v>
       </c>
       <c r="F30" t="str">
-        <v>2026-09-04T10:15:52.847Z</v>
+        <v>2026-09-04T11:41:49.858Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: enhance task management with overdue detection and default status handling
- Implemented overdue detection for tasks in the task list and calendar views.
- Added functionality to ensure default statuses are maintained in the database.
- Introduced automatic promotion of PRD tasks to Done based on specific criteria.
- Updated UI components to reflect overdue status visually.
- Enhanced error handling for modifying and deleting default statuses.
</commit_message>
<xml_diff>
--- a/data/taskDB.xlsx
+++ b/data/taskDB.xlsx
@@ -804,7 +804,7 @@
         <v>2026-09-01T07:23:24.979Z</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-09-04T08:58:01.411Z</v>
+        <v>2026-09-04T12:25:20.571Z</v>
       </c>
     </row>
     <row r="3">
@@ -824,7 +824,7 @@
         <v>2026-09-01T07:23:24.981Z</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-09-04T08:58:01.417Z</v>
+        <v>2026-09-04T12:25:20.575Z</v>
       </c>
     </row>
     <row r="4">
@@ -838,13 +838,13 @@
         <v>#22C55E</v>
       </c>
       <c r="D4" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E4" t="str">
         <v>2026-09-01T07:23:24.983Z</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-09-04T11:33:02.517Z</v>
+        <v>2026-09-04T12:25:20.606Z</v>
       </c>
     </row>
     <row r="5">
@@ -864,7 +864,7 @@
         <v>2026-09-01T07:23:24.985Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-04T11:33:02.520Z</v>
+        <v>2026-09-04T12:25:20.598Z</v>
       </c>
     </row>
     <row r="6">
@@ -878,13 +878,13 @@
         <v>#6BB82A</v>
       </c>
       <c r="D6" t="str">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E6" t="str">
         <v>2026-09-01T07:23:24.988Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-04T11:33:02.514Z</v>
+        <v>2026-09-04T12:25:20.613Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: enhance task sorting with new status-based options and timeline comparisons
- Added a new sorting mode for tasks based on their status.
- Implemented functions to determine the next relevant timeline and secondary timeline for tasks.
- Updated the sorting logic to prioritize tasks based on completion status and relevant timelines.
- Enhanced the overall task sorting functionality to improve task management efficiency.
</commit_message>
<xml_diff>
--- a/data/taskDB.xlsx
+++ b/data/taskDB.xlsx
@@ -804,7 +804,7 @@
         <v>2026-09-01T07:23:24.979Z</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-09-04T12:25:20.571Z</v>
+        <v>2026-09-04T12:51:27.047Z</v>
       </c>
     </row>
     <row r="3">
@@ -824,7 +824,7 @@
         <v>2026-09-01T07:23:24.981Z</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-09-04T12:25:20.575Z</v>
+        <v>2026-09-04T12:51:27.053Z</v>
       </c>
     </row>
     <row r="4">
@@ -844,7 +844,7 @@
         <v>2026-09-01T07:23:24.983Z</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-09-04T12:25:20.606Z</v>
+        <v>2026-09-04T12:51:27.066Z</v>
       </c>
     </row>
     <row r="5">
@@ -864,7 +864,7 @@
         <v>2026-09-01T07:23:24.985Z</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-04T12:25:20.598Z</v>
+        <v>2026-09-04T12:51:27.059Z</v>
       </c>
     </row>
     <row r="6">
@@ -884,7 +884,7 @@
         <v>2026-09-01T07:23:24.988Z</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-09-04T12:25:20.613Z</v>
+        <v>2026-09-04T12:51:27.071Z</v>
       </c>
     </row>
   </sheetData>
@@ -1204,7 +1204,7 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M2" t="str">
-        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+        <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
       </c>
       <c r="N2" t="str">
         <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
@@ -1213,7 +1213,7 @@
         <v>2026-09-04T09:22:21.943Z</v>
       </c>
       <c r="P2" t="str">
-        <v>2026-09-04T09:42:39.373Z</v>
+        <v>2026-09-04T12:29:28.753Z</v>
       </c>
     </row>
     <row r="3">
@@ -1254,7 +1254,7 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M3" t="str">
-        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+        <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
       </c>
       <c r="N3" t="str">
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
@@ -1263,7 +1263,7 @@
         <v>2026-09-04T09:24:04.693Z</v>
       </c>
       <c r="P3" t="str">
-        <v>2026-09-04T09:42:32.107Z</v>
+        <v>2026-09-04T12:29:22.917Z</v>
       </c>
     </row>
     <row r="4">
@@ -1304,7 +1304,7 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M4" t="str">
-        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+        <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
       </c>
       <c r="N4" t="str">
         <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
@@ -1313,7 +1313,7 @@
         <v>2026-09-04T09:24:33.365Z</v>
       </c>
       <c r="P4" t="str">
-        <v>2026-09-04T09:42:23.325Z</v>
+        <v>2026-09-04T12:29:18.513Z</v>
       </c>
     </row>
     <row r="5">
@@ -1354,7 +1354,7 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M5" t="str">
-        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+        <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
       </c>
       <c r="N5" t="str">
         <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
@@ -1363,7 +1363,7 @@
         <v>2026-09-04T09:25:10.002Z</v>
       </c>
       <c r="P5" t="str">
-        <v>2026-09-04T09:42:08.479Z</v>
+        <v>2026-09-04T12:29:13.377Z</v>
       </c>
     </row>
     <row r="6">
@@ -1404,7 +1404,7 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M6" t="str">
-        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+        <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
       </c>
       <c r="N6" t="str">
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
@@ -1413,7 +1413,7 @@
         <v>2026-09-04T09:26:00.676Z</v>
       </c>
       <c r="P6" t="str">
-        <v>2026-09-04T09:42:00.055Z</v>
+        <v>2026-09-04T12:29:08.647Z</v>
       </c>
     </row>
     <row r="7">
@@ -1554,7 +1554,7 @@
         <v>5d2ecd1b-19a8-48d6-80c0-6cd3710e19e0</v>
       </c>
       <c r="M9" t="str">
-        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+        <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
       </c>
       <c r="N9" t="str">
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
@@ -1563,7 +1563,7 @@
         <v>2026-09-04T09:32:18.156Z</v>
       </c>
       <c r="P9" t="str">
-        <v>2026-09-04T09:41:51.999Z</v>
+        <v>2026-09-04T12:29:03.482Z</v>
       </c>
     </row>
     <row r="10">
@@ -2075,7 +2075,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I40"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3063,9 +3063,183 @@
         <v>2026-09-04T11:32:35.136Z</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>f646fb2a-3c6e-4348-857e-44536a0600fd</v>
+      </c>
+      <c r="B35" t="str">
+        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
+      </c>
+      <c r="C35" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="D35" t="str">
+        <v>PRD</v>
+      </c>
+      <c r="E35" t="str">
+        <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Done</v>
+      </c>
+      <c r="G35" t="str">
+        <v>2026-09-04T12:29:03.450Z</v>
+      </c>
+      <c r="H35" t="str">
+        <v>2026-09-04T12:29:03.453Z</v>
+      </c>
+      <c r="I35" t="str">
+        <v>2026-09-04T12:29:03.453Z</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>ae96bf66-08b8-4f0d-ade9-9555df41630f</v>
+      </c>
+      <c r="B36" t="str">
+        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
+      </c>
+      <c r="C36" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="D36" t="str">
+        <v>PRD</v>
+      </c>
+      <c r="E36" t="str">
+        <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Done</v>
+      </c>
+      <c r="G36" t="str">
+        <v>2026-09-04T12:29:08.616Z</v>
+      </c>
+      <c r="H36" t="str">
+        <v>2026-09-04T12:29:08.619Z</v>
+      </c>
+      <c r="I36" t="str">
+        <v>2026-09-04T12:29:08.619Z</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>f8632a7d-ab32-44de-9056-4e40cd2b8ae6</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
+      </c>
+      <c r="C37" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="D37" t="str">
+        <v>PRD</v>
+      </c>
+      <c r="E37" t="str">
+        <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Done</v>
+      </c>
+      <c r="G37" t="str">
+        <v>2026-09-04T12:29:13.347Z</v>
+      </c>
+      <c r="H37" t="str">
+        <v>2026-09-04T12:29:13.349Z</v>
+      </c>
+      <c r="I37" t="str">
+        <v>2026-09-04T12:29:13.349Z</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>f28a93e8-a834-42d7-bc17-b6e2292565a5</v>
+      </c>
+      <c r="B38" t="str">
+        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
+      </c>
+      <c r="C38" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="D38" t="str">
+        <v>PRD</v>
+      </c>
+      <c r="E38" t="str">
+        <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Done</v>
+      </c>
+      <c r="G38" t="str">
+        <v>2026-09-04T12:29:18.482Z</v>
+      </c>
+      <c r="H38" t="str">
+        <v>2026-09-04T12:29:18.485Z</v>
+      </c>
+      <c r="I38" t="str">
+        <v>2026-09-04T12:29:18.485Z</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>54faaead-668f-490e-90b4-f54dd4c8a28e</v>
+      </c>
+      <c r="B39" t="str">
+        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
+      </c>
+      <c r="C39" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="D39" t="str">
+        <v>PRD</v>
+      </c>
+      <c r="E39" t="str">
+        <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Done</v>
+      </c>
+      <c r="G39" t="str">
+        <v>2026-09-04T12:29:22.894Z</v>
+      </c>
+      <c r="H39" t="str">
+        <v>2026-09-04T12:29:22.895Z</v>
+      </c>
+      <c r="I39" t="str">
+        <v>2026-09-04T12:29:22.895Z</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>720dcdc9-3017-46d6-996d-dc96efbfcc9b</v>
+      </c>
+      <c r="B40" t="str">
+        <v>d6acd7ea-e69f-4894-9ce4-c8ae86da6bd2</v>
+      </c>
+      <c r="C40" t="str">
+        <v>3e73c046-732a-4718-80a5-242e8835c1c0</v>
+      </c>
+      <c r="D40" t="str">
+        <v>PRD</v>
+      </c>
+      <c r="E40" t="str">
+        <v>e475d16a-9163-4793-b90e-9aed0ce0e9ec</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Done</v>
+      </c>
+      <c r="G40" t="str">
+        <v>2026-09-04T12:29:28.729Z</v>
+      </c>
+      <c r="H40" t="str">
+        <v>2026-09-04T12:29:28.731Z</v>
+      </c>
+      <c r="I40" t="str">
+        <v>2026-09-04T12:29:28.731Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I40"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3457,10 +3631,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>80990267-d989-453d-b6c0-934f6d17265e</v>
+        <v>f8edc8fa-0fc6-44c4-a15c-14cfe4475d9e</v>
       </c>
       <c r="B8" t="str">
-        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
+        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
       </c>
       <c r="C8" t="str">
         <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
@@ -3469,98 +3643,98 @@
         <v>0</v>
       </c>
       <c r="E8" t="str">
-        <v>2026-09-04T09:41:51.988Z</v>
+        <v>2026-09-04T09:44:49.319Z</v>
       </c>
       <c r="F8" t="str">
-        <v>2026-09-04T09:41:51.988Z</v>
+        <v>2026-09-04T09:44:49.319Z</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>3f788bfd-4196-4334-b70e-e7d4f9aea927</v>
+        <v>e1211e67-dde9-4873-a96f-6985e7753170</v>
       </c>
       <c r="B9" t="str">
-        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
+        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
       </c>
       <c r="C9" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D9" t="str">
         <v>1</v>
       </c>
       <c r="E9" t="str">
-        <v>2026-09-04T09:41:51.994Z</v>
+        <v>2026-09-04T09:44:49.325Z</v>
       </c>
       <c r="F9" t="str">
-        <v>2026-09-04T09:41:51.994Z</v>
+        <v>2026-09-04T09:44:49.325Z</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>32c5e74c-e29b-49ce-8bb9-05c45ae2b05c</v>
+        <v>5a79cab4-c5b3-4c96-8b5a-bf72005b39f2</v>
       </c>
       <c r="B10" t="str">
-        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
+        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
       </c>
       <c r="C10" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D10" t="str">
         <v>0</v>
       </c>
       <c r="E10" t="str">
-        <v>2026-09-04T09:42:00.043Z</v>
+        <v>2026-09-04T09:45:22.504Z</v>
       </c>
       <c r="F10" t="str">
-        <v>2026-09-04T09:42:00.043Z</v>
+        <v>2026-09-04T09:45:22.504Z</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>bc2310d5-a861-4446-b827-d5ca714102c1</v>
+        <v>e16d77fc-e33d-4c73-be58-b8a0016c902a</v>
       </c>
       <c r="B11" t="str">
-        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
+        <v>12f8c884-7a9e-4086-8352-ace2ea778248</v>
       </c>
       <c r="C11" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="D11" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" t="str">
-        <v>2026-09-04T09:42:00.049Z</v>
+        <v>2026-09-04T09:45:31.784Z</v>
       </c>
       <c r="F11" t="str">
-        <v>2026-09-04T09:42:00.049Z</v>
+        <v>2026-09-04T09:45:31.784Z</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>aa0c90a1-50a9-467e-aeff-a80e364d7231</v>
+        <v>76c55ffd-5c72-475c-9448-e969b036b7c0</v>
       </c>
       <c r="B12" t="str">
-        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
+        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
       </c>
       <c r="C12" t="str">
-        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D12" t="str">
         <v>0</v>
       </c>
       <c r="E12" t="str">
-        <v>2026-09-04T09:42:08.465Z</v>
+        <v>2026-09-04T09:47:39.835Z</v>
       </c>
       <c r="F12" t="str">
-        <v>2026-09-04T09:42:08.465Z</v>
+        <v>2026-09-04T09:47:39.835Z</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>64fe364b-f395-498f-8813-6c1bba29fbc3</v>
+        <v>689f964d-b216-40de-881b-605919cf6b35</v>
       </c>
       <c r="B13" t="str">
-        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
+        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
       </c>
       <c r="C13" t="str">
         <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
@@ -3569,38 +3743,38 @@
         <v>1</v>
       </c>
       <c r="E13" t="str">
-        <v>2026-09-04T09:42:08.473Z</v>
+        <v>2026-09-04T09:47:39.839Z</v>
       </c>
       <c r="F13" t="str">
-        <v>2026-09-04T09:42:08.473Z</v>
+        <v>2026-09-04T09:47:39.839Z</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>1df7c234-174e-4ecc-86df-402763448af7</v>
+        <v>be30c4c5-9550-4b85-8401-c243a2cc9973</v>
       </c>
       <c r="B14" t="str">
-        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
+        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
       </c>
       <c r="C14" t="str">
-        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D14" t="str">
         <v>0</v>
       </c>
       <c r="E14" t="str">
-        <v>2026-09-04T09:42:23.314Z</v>
+        <v>2026-09-04T09:48:58.065Z</v>
       </c>
       <c r="F14" t="str">
-        <v>2026-09-04T09:42:23.314Z</v>
+        <v>2026-09-04T09:48:58.065Z</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2c5c97cc-6f06-4a34-b426-104fc1ef7003</v>
+        <v>6402d1cb-71a9-4249-9e8d-765a6d771490</v>
       </c>
       <c r="B15" t="str">
-        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
+        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
       </c>
       <c r="C15" t="str">
         <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
@@ -3609,310 +3783,310 @@
         <v>1</v>
       </c>
       <c r="E15" t="str">
-        <v>2026-09-04T09:42:23.320Z</v>
+        <v>2026-09-04T09:48:58.069Z</v>
       </c>
       <c r="F15" t="str">
-        <v>2026-09-04T09:42:23.320Z</v>
+        <v>2026-09-04T09:48:58.069Z</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>c2f765ad-b590-49db-b0a7-36e85e5895b4</v>
+        <v>837b7f6d-8aa7-4477-a101-2bc781f457eb</v>
       </c>
       <c r="B16" t="str">
-        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
+        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
       </c>
       <c r="C16" t="str">
-        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="D16" t="str">
         <v>0</v>
       </c>
       <c r="E16" t="str">
-        <v>2026-09-04T09:42:32.095Z</v>
+        <v>2026-09-04T10:15:31.431Z</v>
       </c>
       <c r="F16" t="str">
-        <v>2026-09-04T09:42:32.095Z</v>
+        <v>2026-09-04T10:15:31.431Z</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>08a90228-bb97-418f-ac22-e80a3ba6b2cb</v>
+        <v>7bac2115-77f1-401f-ba0e-824e6d60f4fd</v>
       </c>
       <c r="B17" t="str">
-        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
+        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
       </c>
       <c r="C17" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
       </c>
       <c r="D17" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17" t="str">
-        <v>2026-09-04T09:42:32.102Z</v>
+        <v>2026-09-04T10:15:52.847Z</v>
       </c>
       <c r="F17" t="str">
-        <v>2026-09-04T09:42:32.102Z</v>
+        <v>2026-09-04T10:15:52.847Z</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>9c12a7a8-f6ed-48d7-bd22-3b59c5cada75</v>
+        <v>4e27d0ea-d725-4fd6-8af3-af70d286f196</v>
       </c>
       <c r="B18" t="str">
-        <v>d6acd7ea-e69f-4894-9ce4-c8ae86da6bd2</v>
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
       </c>
       <c r="C18" t="str">
-        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
+        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
       </c>
       <c r="D18" t="str">
         <v>0</v>
       </c>
       <c r="E18" t="str">
-        <v>2026-09-04T09:42:39.367Z</v>
+        <v>2026-09-04T11:41:49.851Z</v>
       </c>
       <c r="F18" t="str">
-        <v>2026-09-04T09:42:39.367Z</v>
+        <v>2026-09-04T11:41:49.851Z</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>f8edc8fa-0fc6-44c4-a15c-14cfe4475d9e</v>
+        <v>9c21d982-7ad7-4a32-8875-f8af532fdf47</v>
       </c>
       <c r="B19" t="str">
-        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
+        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
       </c>
       <c r="C19" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D19" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="str">
-        <v>2026-09-04T09:44:49.319Z</v>
+        <v>2026-09-04T11:41:49.858Z</v>
       </c>
       <c r="F19" t="str">
-        <v>2026-09-04T09:44:49.319Z</v>
+        <v>2026-09-04T11:41:49.858Z</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>e1211e67-dde9-4873-a96f-6985e7753170</v>
+        <v>61cb483a-a74d-4d8f-b675-5383b14f8f77</v>
       </c>
       <c r="B20" t="str">
-        <v>58f112bb-1a6e-4e26-8d8a-9bcd3e5bc31d</v>
+        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
       </c>
       <c r="C20" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D20" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20" t="str">
-        <v>2026-09-04T09:44:49.325Z</v>
+        <v>2026-09-04T12:29:03.469Z</v>
       </c>
       <c r="F20" t="str">
-        <v>2026-09-04T09:44:49.325Z</v>
+        <v>2026-09-04T12:29:03.469Z</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>5a79cab4-c5b3-4c96-8b5a-bf72005b39f2</v>
+        <v>fe14404c-70ae-4023-afd5-86198706c46a</v>
       </c>
       <c r="B21" t="str">
-        <v>6ac09b86-b7ee-4b62-b048-4594eca71b6c</v>
+        <v>efd54252-a5fb-4a92-ae20-141a96834757</v>
       </c>
       <c r="C21" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D21" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E21" t="str">
-        <v>2026-09-04T09:45:22.504Z</v>
+        <v>2026-09-04T12:29:03.477Z</v>
       </c>
       <c r="F21" t="str">
-        <v>2026-09-04T09:45:22.504Z</v>
+        <v>2026-09-04T12:29:03.477Z</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>e16d77fc-e33d-4c73-be58-b8a0016c902a</v>
+        <v>5d381f35-c77e-4b8f-a9e7-4cbd4a8a52e8</v>
       </c>
       <c r="B22" t="str">
-        <v>12f8c884-7a9e-4086-8352-ace2ea778248</v>
+        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
       </c>
       <c r="C22" t="str">
-        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
       </c>
       <c r="D22" t="str">
         <v>0</v>
       </c>
       <c r="E22" t="str">
-        <v>2026-09-04T09:45:31.784Z</v>
+        <v>2026-09-04T12:29:08.635Z</v>
       </c>
       <c r="F22" t="str">
-        <v>2026-09-04T09:45:31.784Z</v>
+        <v>2026-09-04T12:29:08.635Z</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>76c55ffd-5c72-475c-9448-e969b036b7c0</v>
+        <v>13efe219-b0c8-4dd9-82ca-e72d52723c88</v>
       </c>
       <c r="B23" t="str">
-        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
+        <v>b5647f0e-4c20-454b-b334-30c5458df783</v>
       </c>
       <c r="C23" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D23" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" t="str">
-        <v>2026-09-04T09:47:39.835Z</v>
+        <v>2026-09-04T12:29:08.641Z</v>
       </c>
       <c r="F23" t="str">
-        <v>2026-09-04T09:47:39.835Z</v>
+        <v>2026-09-04T12:29:08.641Z</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>689f964d-b216-40de-881b-605919cf6b35</v>
+        <v>cff700c0-46bf-44de-83d8-60c73d4565d6</v>
       </c>
       <c r="B24" t="str">
-        <v>e5a48211-b75f-4be3-aeee-dde8da731c1e</v>
+        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
       </c>
       <c r="C24" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
       <c r="D24" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E24" t="str">
-        <v>2026-09-04T09:47:39.839Z</v>
+        <v>2026-09-04T12:29:13.365Z</v>
       </c>
       <c r="F24" t="str">
-        <v>2026-09-04T09:47:39.839Z</v>
+        <v>2026-09-04T12:29:13.365Z</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>be30c4c5-9550-4b85-8401-c243a2cc9973</v>
+        <v>db8acf76-4830-485d-9ee7-4300a8abc346</v>
       </c>
       <c r="B25" t="str">
-        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
+        <v>2982e690-f17b-4b39-8695-ca1ad2d39f5e</v>
       </c>
       <c r="C25" t="str">
-        <v>cb4b5eb4-e713-4a8b-9c9f-680ccdbb70f5</v>
+        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
       </c>
       <c r="D25" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" t="str">
-        <v>2026-09-04T09:48:58.065Z</v>
+        <v>2026-09-04T12:29:13.371Z</v>
       </c>
       <c r="F25" t="str">
-        <v>2026-09-04T09:48:58.065Z</v>
+        <v>2026-09-04T12:29:13.371Z</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>6402d1cb-71a9-4249-9e8d-765a6d771490</v>
+        <v>a0bde16c-883f-435d-a1e6-3ff8173e27fc</v>
       </c>
       <c r="B26" t="str">
-        <v>2ee76ad4-4c3e-40be-9b97-9100e95fa1a7</v>
+        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
       </c>
       <c r="C26" t="str">
-        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="D26" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E26" t="str">
-        <v>2026-09-04T09:48:58.069Z</v>
+        <v>2026-09-04T12:29:18.501Z</v>
       </c>
       <c r="F26" t="str">
-        <v>2026-09-04T09:48:58.069Z</v>
+        <v>2026-09-04T12:29:18.501Z</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>837b7f6d-8aa7-4477-a101-2bc781f457eb</v>
+        <v>35763cf5-1687-4782-a94f-47223bc94f62</v>
       </c>
       <c r="B27" t="str">
-        <v>e49e5c13-9c33-449b-9c2c-3b48f3119d16</v>
+        <v>b1e061e4-cef5-46b4-a149-31d4340bd038</v>
       </c>
       <c r="C27" t="str">
-        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D27" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" t="str">
-        <v>2026-09-04T10:15:31.431Z</v>
+        <v>2026-09-04T12:29:18.507Z</v>
       </c>
       <c r="F27" t="str">
-        <v>2026-09-04T10:15:31.431Z</v>
+        <v>2026-09-04T12:29:18.507Z</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>7bac2115-77f1-401f-ba0e-824e6d60f4fd</v>
+        <v>035c1398-3263-4e99-8273-9aba0c9023ba</v>
       </c>
       <c r="B28" t="str">
-        <v>e323d9c8-295f-472c-93f3-fefc39655d80</v>
+        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
       </c>
       <c r="C28" t="str">
-        <v>8e355007-1776-4861-bb6a-5b2e9447c100</v>
+        <v>6fc8b803-c4b5-4da4-8c0c-ce22db0bb86b</v>
       </c>
       <c r="D28" t="str">
         <v>0</v>
       </c>
       <c r="E28" t="str">
-        <v>2026-09-04T10:15:52.847Z</v>
+        <v>2026-09-04T12:29:22.908Z</v>
       </c>
       <c r="F28" t="str">
-        <v>2026-09-04T10:15:52.847Z</v>
+        <v>2026-09-04T12:29:22.908Z</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>4e27d0ea-d725-4fd6-8af3-af70d286f196</v>
+        <v>544f63ce-d992-4c80-aaac-33a8fa860614</v>
       </c>
       <c r="B29" t="str">
-        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+        <v>764fd6d8-3712-4019-8c67-6e3615085faf</v>
       </c>
       <c r="C29" t="str">
-        <v>d19889fc-d565-477e-aa2e-79d7fd239b53</v>
+        <v>5c481da1-0976-4a6d-93ea-b54c40d0ed4f</v>
       </c>
       <c r="D29" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" t="str">
-        <v>2026-09-04T11:41:49.851Z</v>
+        <v>2026-09-04T12:29:22.912Z</v>
       </c>
       <c r="F29" t="str">
-        <v>2026-09-04T11:41:49.851Z</v>
+        <v>2026-09-04T12:29:22.912Z</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>9c21d982-7ad7-4a32-8875-f8af532fdf47</v>
+        <v>5da43984-fa10-419d-be97-55c04f991d54</v>
       </c>
       <c r="B30" t="str">
-        <v>81722c13-7a3f-4789-a1ac-a70c472369e0</v>
+        <v>d6acd7ea-e69f-4894-9ce4-c8ae86da6bd2</v>
       </c>
       <c r="C30" t="str">
-        <v>4e0d447b-431f-4ad8-9dcc-39bf5a30dd6b</v>
+        <v>55d6e756-c40c-4755-84ab-c3458437acd6</v>
       </c>
       <c r="D30" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E30" t="str">
-        <v>2026-09-04T11:41:49.858Z</v>
+        <v>2026-09-04T12:29:28.748Z</v>
       </c>
       <c r="F30" t="str">
-        <v>2026-09-04T11:41:49.858Z</v>
+        <v>2026-09-04T12:29:28.748Z</v>
       </c>
     </row>
   </sheetData>

</xml_diff>